<commit_message>
feat: update single service structure
</commit_message>
<xml_diff>
--- a/parsing/data/services-import.xlsx
+++ b/parsing/data/services-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:T43"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,21 +419,45 @@
         <v>category</v>
       </c>
       <c r="G1" t="str">
+        <v>image</v>
+      </c>
+      <c r="H1" t="str">
+        <v>price_main</v>
+      </c>
+      <c r="I1" t="str">
+        <v>price_extra</v>
+      </c>
+      <c r="J1" t="str">
+        <v>price_diagnostics</v>
+      </c>
+      <c r="K1" t="str">
+        <v>warranty_text</v>
+      </c>
+      <c r="L1" t="str">
+        <v>related_brands</v>
+      </c>
+      <c r="M1" t="str">
+        <v>faq_title</v>
+      </c>
+      <c r="N1" t="str">
+        <v>faq</v>
+      </c>
+      <c r="O1" t="str">
         <v>Focus Keyword</v>
       </c>
-      <c r="H1" t="str">
+      <c r="P1" t="str">
         <v>SEO Title</v>
       </c>
-      <c r="I1" t="str">
+      <c r="Q1" t="str">
         <v>Meta Description</v>
       </c>
-      <c r="J1" t="str">
+      <c r="R1" t="str">
         <v>Meta Keywords</v>
       </c>
-      <c r="K1" t="str">
+      <c r="S1" t="str">
         <v>Facebook Title</v>
       </c>
-      <c r="L1" t="str">
+      <c r="T1" t="str">
         <v>Twitter Title</v>
       </c>
     </row>
@@ -457,21 +481,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G2" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/biled.jpg</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 8 500 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L2" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Сколько времени занимает замена линз в фарах?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 8 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O2" t="str">
         <v>установка линз</v>
       </c>
-      <c r="H2" t="str">
+      <c r="P2" t="str">
         <v>Установка линз (Xenon/Bi-LED) в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I2" t="str">
+      <c r="Q2" t="str">
         <v>Меняем выгоревшие линзы на модули Xenon или Bi-LED. Цена от 8 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J2" t="str">
+      <c r="R2" t="str">
         <v>установка линз, установка линз спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K2" t="str">
+      <c r="S2" t="str">
         <v>Установка линз (Xenon/Bi-LED) в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L2" t="str">
+      <c r="T2" t="str">
         <v>Установка линз (Xenon/Bi-LED) в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -495,21 +543,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G3" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/YYAAAgDI0OA-960.jpg</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка лазерных модулей::от 35 000 ₽ / шт.::3-5 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L3" t="str">
+        <v>BMW|MERCEDES|AUDI|LEXUS|PORSCHE|Land Rover|JAGUAR|INFINITI|Maserati|BENTLEY</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Сколько времени занимает установка лазерных?::Установка лазерных модулей — обычно 3–5 часов.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 35 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O3" t="str">
         <v>установка лазерных</v>
       </c>
-      <c r="H3" t="str">
+      <c r="P3" t="str">
         <v>Установка лазерных (Laser) линз в СПб — от 35 000 ₽ | КБ АВ…</v>
       </c>
-      <c r="I3" t="str">
+      <c r="Q3" t="str">
         <v>Топовые лазерные модули с дальним светом до 600 м. Для тех, кто хочет максимум. Цена от 35 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J3" t="str">
+      <c r="R3" t="str">
         <v>установка лазерных, установка лазерных спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K3" t="str">
+      <c r="S3" t="str">
         <v>Установка лазерных (Laser) линз в СПб — от 35 000 ₽ | КБ АВ…</v>
       </c>
-      <c r="L3" t="str">
+      <c r="T3" t="str">
         <v>Установка лазерных (Laser) линз в СПб — от 35 000 ₽ | КБ АВ…</v>
       </c>
     </row>
@@ -533,21 +605,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G4" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/polish-1.jpg</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Шлифовка и полировка стекла::от 2 500 ₽::1-2 ч::6 мес.|Защитное покрытие::входит в стоимость::30 мин::-</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Полировка изнутри (при разборке)::от 1 500 ₽::+1 ч::1 год|Устранение глубоких царапин::от 1 000 ₽::+1 ч::-</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L4" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Сколько времени занимает полировка и шлифовка фар?::Обычно 1–2 часа на пару фар.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O4" t="str">
         <v>полировка и шлифовка фар</v>
       </c>
-      <c r="H4" t="str">
+      <c r="P4" t="str">
         <v>Полировка и шлифовка фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I4" t="str">
+      <c r="Q4" t="str">
         <v>Глубокая шлифовка и полировка — возвращаем прозрачность без замены стекла. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J4" t="str">
+      <c r="R4" t="str">
         <v>полировка и шлифовка фар, полировка и шлифовка фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K4" t="str">
+      <c r="S4" t="str">
         <v>Полировка и шлифовка фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L4" t="str">
+      <c r="T4" t="str">
         <v>Полировка и шлифовка фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -571,21 +667,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G5" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/8FeX41yZ3b2mVdd1jWi45NW5uoY-960.jpg</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 2 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L5" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Сколько времени занимает ремонт фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O5" t="str">
         <v>ремонт фар</v>
       </c>
-      <c r="H5" t="str">
+      <c r="P5" t="str">
         <v>Ремонт фар (комплексный) в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I5" t="str">
+      <c r="Q5" t="str">
         <v>Восстанавливаем фары после ДТП, заливов и выгорания LED. От галогена до лазерных модулей. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J5" t="str">
+      <c r="R5" t="str">
         <v>ремонт фар, ремонт фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K5" t="str">
+      <c r="S5" t="str">
         <v>Ремонт фар (комплексный) в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L5" t="str">
+      <c r="T5" t="str">
         <v>Ремонт фар (комплексный) в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -609,21 +729,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G6" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/08/img_6069.jpg</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена стекла фары::от 5 000 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L6" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Сколько времени занимает замена стёкол фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O6" t="str">
         <v>замена стёкол фар</v>
       </c>
-      <c r="H6" t="str">
+      <c r="P6" t="str">
         <v>Замена стёкол фар в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I6" t="str">
+      <c r="Q6" t="str">
         <v>Демонтируем треснувшее или мутное стекло, устанавливаем новое с герметизацией корпуса. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J6" t="str">
+      <c r="R6" t="str">
         <v>замена стёкол фар, замена стёкол фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K6" t="str">
+      <c r="S6" t="str">
         <v>Замена стёкол фар в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L6" t="str">
+      <c r="T6" t="str">
         <v>Замена стёкол фар в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -647,21 +791,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G7" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/misted-1.jpg</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Устранение запотевания и просушка::от 3 500 ₽::2-3 ч::1 год|Замена уплотнителя / клапанов::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L7" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Сколько времени занимает устранение запотевания фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O7" t="str">
         <v>устранение запотевания фар</v>
       </c>
-      <c r="H7" t="str">
+      <c r="P7" t="str">
         <v>Устранение запотевания фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I7" t="str">
+      <c r="Q7" t="str">
         <v>Диагностируем причину, переклеиваем корпус по заводским технологиям. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J7" t="str">
+      <c r="R7" t="str">
         <v>устранение запотевания фар, устранение запотевания фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K7" t="str">
+      <c r="S7" t="str">
         <v>Устранение запотевания фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L7" t="str">
+      <c r="T7" t="str">
         <v>Устранение запотевания фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -685,21 +853,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G8" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-36.jpg</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 8 500 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L8" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Сколько времени занимает установка bi-led?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 8 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O8" t="str">
         <v>установка bi-led линз</v>
       </c>
-      <c r="H8" t="str">
+      <c r="P8" t="str">
         <v>Установка Bi-LED линз в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I8" t="str">
+      <c r="Q8" t="str">
         <v>Переходим на качественный диодный свет. Ярче ксенона, без слепящего встречного потока. Цена от 8 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J8" t="str">
+      <c r="R8" t="str">
         <v>установка bi-led линз, установка bi-led линз спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K8" t="str">
+      <c r="S8" t="str">
         <v>Установка Bi-LED линз в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L8" t="str">
+      <c r="T8" t="str">
         <v>Установка Bi-LED линз в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -723,21 +915,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G9" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/xenon.jpg</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка ксенонового комплекта::от 5 000 ₽::2-4 ч::1 год|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L9" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Сколько времени занимает установка ксенона?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O9" t="str">
         <v>установка ксенона</v>
       </c>
-      <c r="H9" t="str">
+      <c r="P9" t="str">
         <v>Установка ксенона (штатные комплекты) в СПб — от 5 000 ₽ |…</v>
       </c>
-      <c r="I9" t="str">
+      <c r="Q9" t="str">
         <v>Монтируем штатные ксеноновые комплекты с правильной фокусировкой и герметизацией. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J9" t="str">
+      <c r="R9" t="str">
         <v>установка ксенона, установка ксенона спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K9" t="str">
+      <c r="S9" t="str">
         <v>Установка ксенона (штатные комплекты) в СПб — от 5 000 ₽ |…</v>
       </c>
-      <c r="L9" t="str">
+      <c r="T9" t="str">
         <v>Установка ксенона (штатные комплекты) в СПб — от 5 000 ₽ |…</v>
       </c>
     </row>
@@ -761,21 +977,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G10" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/09/F4AAAgKEmOA-960.jpg</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 6 000 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L10" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Сколько времени занимает замена штатных линз на оригинал или аналог?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O10" t="str">
         <v>замена штатных линз на оригинал/аналог</v>
       </c>
-      <c r="H10" t="str">
+      <c r="P10" t="str">
         <v>Замена штатных линз на оригинал/аналог в СПб — от 6 000 ₽ |…</v>
       </c>
-      <c r="I10" t="str">
+      <c r="Q10" t="str">
         <v>Меняем заводские линзы на оригинал или проверенный аналог с настройкой света. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J10" t="str">
+      <c r="R10" t="str">
         <v>замена штатных линз на оригинал/аналог, замена штатных линз на оригинал/аналог спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K10" t="str">
+      <c r="S10" t="str">
         <v>Замена штатных линз на оригинал/аналог в СПб — от 6 000 ₽ |…</v>
       </c>
-      <c r="L10" t="str">
+      <c r="T10" t="str">
         <v>Замена штатных линз на оригинал/аналог в СПб — от 6 000 ₽ |…</v>
       </c>
     </row>
@@ -799,21 +1039,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G11" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/5141ad6393277.jpeg</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 2 500 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L11" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Сколько времени занимает тюнинг подсветки?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O11" t="str">
         <v>тюнинг подсветки</v>
       </c>
-      <c r="H11" t="str">
+      <c r="P11" t="str">
         <v>Тюнинг подсветки (Ангельские/Дьявольские глазки) в СПб — от…</v>
       </c>
-      <c r="I11" t="str">
+      <c r="Q11" t="str">
         <v>Устанавливаем ангельские и дьявольские глазки с аккуратной проводкой и герметизацией. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J11" t="str">
+      <c r="R11" t="str">
         <v>тюнинг подсветки, тюнинг подсветки спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K11" t="str">
+      <c r="S11" t="str">
         <v>Тюнинг подсветки (Ангельские/Дьявольские глазки) в СПб — от…</v>
       </c>
-      <c r="L11" t="str">
+      <c r="T11" t="str">
         <v>Тюнинг подсветки (Ангельские/Дьявольские глазки) в СПб — от…</v>
       </c>
     </row>
@@ -837,21 +1101,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G12" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/paint.png</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Покраска масок фар::от 3 500 ₽::1 день::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Покраска декоративных элементов::от 1 500 ₽::+4 ч::-|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L12" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Сколько времени занимает покраска масок фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O12" t="str">
         <v>покраска масок фар</v>
       </c>
-      <c r="H12" t="str">
+      <c r="P12" t="str">
         <v>Покраска масок фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I12" t="str">
+      <c r="Q12" t="str">
         <v>Красим внутренние маски термостойкой краской — чёрный, хром или под ваш стиль. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J12" t="str">
+      <c r="R12" t="str">
         <v>покраска масок фар, покраска масок фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K12" t="str">
+      <c r="S12" t="str">
         <v>Покраска масок фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L12" t="str">
+      <c r="T12" t="str">
         <v>Покраска масок фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -875,21 +1163,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G13" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/kyaaagkceoa-960.jpg</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 5 000 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L13" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Сколько времени занимает изготовление дневных ходовых огней?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O13" t="str">
         <v>изготовление дхо</v>
       </c>
-      <c r="H13" t="str">
+      <c r="P13" t="str">
         <v>Изготовление ДХО в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I13" t="str">
+      <c r="Q13" t="str">
         <v>Делаем индивидуальные ДХО под вашу оптику с заводской герметичностью. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J13" t="str">
+      <c r="R13" t="str">
         <v>изготовление дхо, изготовление дхо спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K13" t="str">
+      <c r="S13" t="str">
         <v>Изготовление ДХО в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L13" t="str">
+      <c r="T13" t="str">
         <v>Изготовление ДХО в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -913,21 +1225,45 @@
         <v>Регулировка и диагностика</v>
       </c>
       <c r="G14" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/reg.jpg</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Регулировка на оптическом стенде::от 2 000 ₽::30-60 мин::-</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Диагностика оптики перед регулировкой::Бесплатно::+15 мин::-</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Проверка светового пучка::Входит в стоимость::15 мин::-</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L14" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Сколько времени занимает регулировка света фар на оптическом стенде?::Регулировка занимает 30–60 минут.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
+      </c>
+      <c r="O14" t="str">
         <v>регулировка света на стенде</v>
       </c>
-      <c r="H14" t="str">
+      <c r="P14" t="str">
         <v>Регулировка света на стенде в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I14" t="str">
+      <c r="Q14" t="str">
         <v>Выставляем правильный световой пучок на стенде — без слепящего встречного. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J14" t="str">
+      <c r="R14" t="str">
         <v>регулировка света на стенде, регулировка света на стенде спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K14" t="str">
+      <c r="S14" t="str">
         <v>Регулировка света на стенде в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L14" t="str">
+      <c r="T14" t="str">
         <v>Регулировка света на стенде в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -951,21 +1287,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G15" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/aeecc8es-960-1.jpg</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 2 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L15" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Сколько времени занимает замена штатных блоков розжига и ламп?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O15" t="str">
         <v>замена блоков розжига и ламп</v>
       </c>
-      <c r="H15" t="str">
+      <c r="P15" t="str">
         <v>Замена блоков розжига и ламп в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I15" t="str">
+      <c r="Q15" t="str">
         <v>Меняем блоки розжига и лампы, проверяем всю цепь ксенона. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J15" t="str">
+      <c r="R15" t="str">
         <v>замена блоков розжига и ламп, замена блоков розжига и ламп спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K15" t="str">
+      <c r="S15" t="str">
         <v>Замена блоков розжига и ламп в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L15" t="str">
+      <c r="T15" t="str">
         <v>Замена блоков розжига и ламп в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -989,21 +1349,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G16" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/drQAAgC09-A-9601.jpg</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 3 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L16" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Сколько времени занимает ремонт штатных дхо?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O16" t="str">
         <v>ремонт штатных дхо</v>
       </c>
-      <c r="H16" t="str">
+      <c r="P16" t="str">
         <v>Ремонт штатных ДХО в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I16" t="str">
+      <c r="Q16" t="str">
         <v>Компонентно восстанавливаем штатные дневные ходовые огни. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J16" t="str">
+      <c r="R16" t="str">
         <v>ремонт штатных дхо, ремонт штатных дхо спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K16" t="str">
+      <c r="S16" t="str">
         <v>Ремонт штатных ДХО в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L16" t="str">
+      <c r="T16" t="str">
         <v>Ремонт штатных ДХО в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1027,21 +1411,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G17" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/MAAAgENOOA-19201.jpg</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 4 000 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L17" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Сколько времени занимает установка динамических?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O17" t="str">
         <v>динамические</v>
       </c>
-      <c r="H17" t="str">
+      <c r="P17" t="str">
         <v>Динамические («бегущие») поворотники в СПб — от 4 000 ₽ | К…</v>
       </c>
-      <c r="I17" t="str">
+      <c r="Q17" t="str">
         <v>Монтируем динамические поворотники с прошивкой или обманками при необходимости. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J17" t="str">
+      <c r="R17" t="str">
         <v>динамические, динамические спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K17" t="str">
+      <c r="S17" t="str">
         <v>Динамические («бегущие») поворотники в СПб — от 4 000 ₽ | К…</v>
       </c>
-      <c r="L17" t="str">
+      <c r="T17" t="str">
         <v>Динамические («бегущие») поворотники в СПб — от 4 000 ₽ | К…</v>
       </c>
     </row>
@@ -1065,21 +1473,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G18" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/06/YoAAAgFugOA-960.jpg</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт светодиодных модулей::от 4 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L18" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Сколько времени занимает ремонт штатных светодиодных фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O18" t="str">
         <v>ремонт светодиодных фар</v>
       </c>
-      <c r="H18" t="str">
+      <c r="P18" t="str">
         <v>Ремонт светодиодных фар (LED) в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I18" t="str">
+      <c r="Q18" t="str">
         <v>Заменяем диоды в неразборных модулях — когда другим не по силам. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J18" t="str">
+      <c r="R18" t="str">
         <v>ремонт светодиодных фар, ремонт светодиодных фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K18" t="str">
+      <c r="S18" t="str">
         <v>Ремонт светодиодных фар (LED) в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L18" t="str">
+      <c r="T18" t="str">
         <v>Ремонт светодиодных фар (LED) в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1103,21 +1535,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G19" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/rear-1.jpg</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт светодиодных модулей::от 3 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L19" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Сколько времени занимает ремонт штатных светодиодных фонарей?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O19" t="str">
         <v>ремонт светодиодных фонарей</v>
       </c>
-      <c r="H19" t="str">
+      <c r="P19" t="str">
         <v>Ремонт светодиодных фонарей (задняя оптика) в СПб — от 3 50…</v>
       </c>
-      <c r="I19" t="str">
+      <c r="Q19" t="str">
         <v>Восстанавливаем заднюю LED-оптику: диоды, платы, драйверы. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J19" t="str">
+      <c r="R19" t="str">
         <v>ремонт светодиодных фонарей, ремонт светодиодных фонарей спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K19" t="str">
+      <c r="S19" t="str">
         <v>Ремонт светодиодных фонарей (задняя оптика) в СПб — от 3 50…</v>
       </c>
-      <c r="L19" t="str">
+      <c r="T19" t="str">
         <v>Ремонт светодиодных фонарей (задняя оптика) в СПб — от 3 50…</v>
       </c>
     </row>
@@ -1141,21 +1597,45 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G20" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/ledfog.png</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Установка ПТФ::от 6 000 ₽::2-4 ч::1 год|Программная активация (при необходимости)::входит в стоимость / от 2 000 ₽::+30-60 мин::-</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Замена стекла / ламп ПТФ::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L20" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Сколько времени занимает установка и программная активация птф?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O20" t="str">
         <v>установка и активация птф</v>
       </c>
-      <c r="H20" t="str">
+      <c r="P20" t="str">
         <v>Установка и активация ПТФ (с прошивкой ЭБУ) в СПб — от 6 00…</v>
       </c>
-      <c r="I20" t="str">
+      <c r="Q20" t="str">
         <v>Монтаж ПТФ под ключ с прошивкой ЭБУ и активацией в меню. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J20" t="str">
+      <c r="R20" t="str">
         <v>установка и активация птф, установка и активация птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K20" t="str">
+      <c r="S20" t="str">
         <v>Установка и активация ПТФ (с прошивкой ЭБУ) в СПб — от 6 00…</v>
       </c>
-      <c r="L20" t="str">
+      <c r="T20" t="str">
         <v>Установка и активация ПТФ (с прошивкой ЭБУ) в СПб — от 6 00…</v>
       </c>
     </row>
@@ -1179,21 +1659,45 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G21" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-35.jpg</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Установка ПТФ::от 5 000 ₽::2-4 ч::1 год|Программная активация (при необходимости)::входит в стоимость / от 2 000 ₽::+30-60 мин::-</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Замена стекла / ламп ПТФ::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L21" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Сколько времени занимает установка светодиодных противотуманных фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O21" t="str">
         <v>установка светодиодных птф</v>
       </c>
-      <c r="H21" t="str">
+      <c r="P21" t="str">
         <v>Установка светодиодных ПТФ в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I21" t="str">
+      <c r="Q21" t="str">
         <v>Ставим LED ПТФ с правильной направленностью и подключением. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J21" t="str">
+      <c r="R21" t="str">
         <v>установка светодиодных птф, установка светодиодных птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K21" t="str">
+      <c r="S21" t="str">
         <v>Установка светодиодных ПТФ в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L21" t="str">
+      <c r="T21" t="str">
         <v>Установка светодиодных ПТФ в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1217,21 +1721,45 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G22" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/s0AAAgHi0OA-960.jpg</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Замена стёкол ПТФ::от 3 000 ₽::30-90 мин::6 мес.</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Полировка стекла ПТФ::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L22" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Сколько времени занимает замена стёкол противотуманных фар?::Замена стёкол ПТФ — обычно до 1,5 часов.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
+      </c>
+      <c r="O22" t="str">
         <v>замена стёкол птф</v>
       </c>
-      <c r="H22" t="str">
+      <c r="P22" t="str">
         <v>Замена стёкол ПТФ в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I22" t="str">
+      <c r="Q22" t="str">
         <v>Меняем треснувшее или мутное стекло ПТФ с герметизацией. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J22" t="str">
+      <c r="R22" t="str">
         <v>замена стёкол птф, замена стёкол птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K22" t="str">
+      <c r="S22" t="str">
         <v>Замена стёкол ПТФ в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L22" t="str">
+      <c r="T22" t="str">
         <v>Замена стёкол ПТФ в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1255,21 +1783,45 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G23" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-8.jpg</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Замена ламп в ПТФ::от 1 500 ₽::30-90 мин::-</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Полировка стекла ПТФ::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L23" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Сколько времени занимает замена ламп в птф?::Работы занимают 30–90 минут.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 1 500 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
+      </c>
+      <c r="O23" t="str">
         <v>замена ламп в птф</v>
       </c>
-      <c r="H23" t="str">
+      <c r="P23" t="str">
         <v>Замена ламп в ПТФ в СПб — от 1 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I23" t="str">
+      <c r="Q23" t="str">
         <v>Быстрая замена ламп в противотуманках с проверкой контактов. Цена от 1 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J23" t="str">
+      <c r="R23" t="str">
         <v>замена ламп в птф, замена ламп в птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K23" t="str">
+      <c r="S23" t="str">
         <v>Замена ламп в ПТФ в СПб — от 1 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L23" t="str">
+      <c r="T23" t="str">
         <v>Замена ламп в ПТФ в СПб — от 1 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1293,21 +1845,45 @@
         <v>Доп. услуги</v>
       </c>
       <c r="G24" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/08/img_3959.jpg</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Замена ламп на светодиодные::от 2 000 ₽::30-90 мин::1 год</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Установка «обманок» (при ошибках в бортовом)::от 500 ₽::+15 мин::-</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L24" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Сколько времени занимает замена ламп на светодиодные?::Замена ламп занимает от 30 минут.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
+      </c>
+      <c r="O24" t="str">
         <v>замена ламп на светодиодные</v>
       </c>
-      <c r="H24" t="str">
+      <c r="P24" t="str">
         <v>Замена ламп на светодиодные (салон, габариты, подсветка ном…</v>
       </c>
-      <c r="I24" t="str">
+      <c r="Q24" t="str">
         <v>Переводим салон, габариты и подсветку номера на качественные LED. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J24" t="str">
+      <c r="R24" t="str">
         <v>замена ламп на светодиодные, замена ламп на светодиодные спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K24" t="str">
+      <c r="S24" t="str">
         <v>Замена ламп на светодиодные (салон, габариты, подсветка ном…</v>
       </c>
-      <c r="L24" t="str">
+      <c r="T24" t="str">
         <v>Замена ламп на светодиодные (салон, габариты, подсветка ном…</v>
       </c>
     </row>
@@ -1331,21 +1907,45 @@
         <v>Механика</v>
       </c>
       <c r="G25" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/e-repair-1.jpg</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Диагностика узла::Входит в стоимость::30 мин::-|Ремонт механики::от 2 500 ₽::1-3 ч::1 год</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Замена узла целиком::по согласованию::+1-2 ч::по запчасти</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L25" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Сколько времени занимает ремонт корректора фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O25" t="str">
         <v>ремонт корректора фар</v>
       </c>
-      <c r="H25" t="str">
+      <c r="P25" t="str">
         <v>Ремонт корректора фар (ручной/авто) в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="I25" t="str">
+      <c r="Q25" t="str">
         <v>Чиним ручные и автоматические корректоры — мотор, тяги, датчики. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J25" t="str">
+      <c r="R25" t="str">
         <v>ремонт корректора фар, ремонт корректора фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K25" t="str">
+      <c r="S25" t="str">
         <v>Ремонт корректора фар (ручной/авто) в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="L25" t="str">
+      <c r="T25" t="str">
         <v>Ремонт корректора фар (ручной/авто) в СПб — от 2 500 ₽ | КБ…</v>
       </c>
     </row>
@@ -1369,21 +1969,45 @@
         <v>Механика</v>
       </c>
       <c r="G26" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/how-to-choose-the-best-car-amplifier.jpg</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Диагностика узла::Входит в стоимость::30 мин::-|Ремонт механики::от 2 000 ₽::1-3 ч::1 год</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Замена узла целиком::по согласованию::+1-2 ч::по запчасти</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L26" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Сколько времени занимает ремонт омывателя фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O26" t="str">
         <v>ремонт омывателя фар</v>
       </c>
-      <c r="H26" t="str">
+      <c r="P26" t="str">
         <v>Ремонт омывателя фар в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I26" t="str">
+      <c r="Q26" t="str">
         <v>Чистим форсунки, ремонтируем насосы и магистрали омывателя. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J26" t="str">
+      <c r="R26" t="str">
         <v>ремонт омывателя фар, ремонт омывателя фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K26" t="str">
+      <c r="S26" t="str">
         <v>Ремонт омывателя фар в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L26" t="str">
+      <c r="T26" t="str">
         <v>Ремонт омывателя фар в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1407,21 +2031,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G27" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/reflector-1.png</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Чистка или замена отражателей::от 6 000 ₽::3-5 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Вакуумное напыление отражателя::от 6 000 ₽::+1 день::1 год|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L27" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Сколько времени занимает ремонт отражателей фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O27" t="str">
         <v>ремонт отражателей / вакуумное напыление</v>
       </c>
-      <c r="H27" t="str">
+      <c r="P27" t="str">
         <v>Ремонт отражателей / вакуумное напыление в СПб — от 6 000 ₽…</v>
       </c>
-      <c r="I27" t="str">
+      <c r="Q27" t="str">
         <v>Чистим, заменяем или восстанавливаем отражатели методом вакуумного напыления — как с завода. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J27" t="str">
+      <c r="R27" t="str">
         <v>ремонт отражателей / вакуумное напыление, ремонт отражателей / вакуумное напыление спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K27" t="str">
+      <c r="S27" t="str">
         <v>Ремонт отражателей / вакуумное напыление в СПб — от 6 000 ₽…</v>
       </c>
-      <c r="L27" t="str">
+      <c r="T27" t="str">
         <v>Ремонт отражателей / вакуумное напыление в СПб — от 6 000 ₽…</v>
       </c>
     </row>
@@ -1445,21 +2093,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G28" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/9AAAAgDfYuA-19201.jpg</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт корпуса фары::от 2 500 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L28" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Сколько времени занимает ремонт корпуса фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O28" t="str">
         <v>ремонт корпуса фар</v>
       </c>
-      <c r="H28" t="str">
+      <c r="P28" t="str">
         <v>Ремонт корпуса фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I28" t="str">
+      <c r="Q28" t="str">
         <v>Герметично восстанавливаем трещины и сколы корпуса фары. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J28" t="str">
+      <c r="R28" t="str">
         <v>ремонт корпуса фар, ремонт корпуса фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K28" t="str">
+      <c r="S28" t="str">
         <v>Ремонт корпуса фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L28" t="str">
+      <c r="T28" t="str">
         <v>Ремонт корпуса фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1483,21 +2155,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G29" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/syAAAgDNyeA-19201.jpg</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Восстановление креплений («ушек»)::от 2 500 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L29" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Сколько времени занимает восстановление креплений?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O29" t="str">
         <v>восстановление креплений</v>
       </c>
-      <c r="H29" t="str">
+      <c r="P29" t="str">
         <v>Восстановление креплений («ушек») в СПб — от 2 500 ₽ | КБ А…</v>
       </c>
-      <c r="I29" t="str">
+      <c r="Q29" t="str">
         <v>Сварка пластика или ремкомплекты — фара снова держится надёжно. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J29" t="str">
+      <c r="R29" t="str">
         <v>восстановление креплений, восстановление креплений спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K29" t="str">
+      <c r="S29" t="str">
         <v>Восстановление креплений («ушек») в СПб — от 2 500 ₽ | КБ А…</v>
       </c>
-      <c r="L29" t="str">
+      <c r="T29" t="str">
         <v>Восстановление креплений («ушек») в СПб — от 2 500 ₽ | КБ А…</v>
       </c>
     </row>
@@ -1521,21 +2217,45 @@
         <v>Механика</v>
       </c>
       <c r="G30" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/6f836g4k337-960.jpg</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 3 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L30" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Сколько времени занимает ремонт ксеноновых фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O30" t="str">
         <v>ремонт ксеноновых фар</v>
       </c>
-      <c r="H30" t="str">
+      <c r="P30" t="str">
         <v>Ремонт ксеноновых фар (спец. узлы) в СПб — от 3 000 ₽ | КБ…</v>
       </c>
-      <c r="I30" t="str">
+      <c r="Q30" t="str">
         <v>Диагностика и ремонт специфических узлов штатного ксенона. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J30" t="str">
+      <c r="R30" t="str">
         <v>ремонт ксеноновых фар, ремонт ксеноновых фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K30" t="str">
+      <c r="S30" t="str">
         <v>Ремонт ксеноновых фар (спец. узлы) в СПб — от 3 000 ₽ | КБ…</v>
       </c>
-      <c r="L30" t="str">
+      <c r="T30" t="str">
         <v>Ремонт ксеноновых фар (спец. узлы) в СПб — от 3 000 ₽ | КБ…</v>
       </c>
     </row>
@@ -1559,21 +2279,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G31" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/QwisvkNREXiXiDRRslmWElJGht4-960.jpg</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 5 000 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L31" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Сколько времени занимает комплексное улучшение света фар?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O31" t="str">
         <v>комплексное улучшение света</v>
       </c>
-      <c r="H31" t="str">
+      <c r="P31" t="str">
         <v>Комплексное улучшение света в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I31" t="str">
+      <c r="Q31" t="str">
         <v>Подбираем оптимальное решение под ваш бюджет и задачи. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J31" t="str">
+      <c r="R31" t="str">
         <v>комплексное улучшение света, комплексное улучшение света спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K31" t="str">
+      <c r="S31" t="str">
         <v>Комплексное улучшение света в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L31" t="str">
+      <c r="T31" t="str">
         <v>Комплексное улучшение света в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1597,21 +2341,45 @@
         <v>Ремонт фар</v>
       </c>
       <c r="G32" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2022/04/S7jUlvfRpkxQN06kpudCI9as0o-960.jpg</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 3 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L32" t="str">
+        <v>BMW|MERCEDES|AUDI|Volkswagen|PORSCHE|VOLVO|Land Rover|JAGUAR|MINI|Skoda|OPEL|PEUGEOT|RENAULT</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Сколько времени занимает ремонт фар европейских производителей?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O32" t="str">
         <v>ремонт фар европейских производителей</v>
       </c>
-      <c r="H32" t="str">
+      <c r="P32" t="str">
         <v>Ремонт фар европейских производителей в СПб — от 3 500 ₽ |…</v>
       </c>
-      <c r="I32" t="str">
+      <c r="Q32" t="str">
         <v>Ремонт и восстановление фар европейских брендов — Valeo, Hella, Bosch, Magneti Marelli и аналоги. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J32" t="str">
+      <c r="R32" t="str">
         <v>ремонт фар европейских производителей, ремонт фар европейских производителей спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K32" t="str">
+      <c r="S32" t="str">
         <v>Ремонт фар европейских производителей в СПб — от 3 500 ₽ |…</v>
       </c>
-      <c r="L32" t="str">
+      <c r="T32" t="str">
         <v>Ремонт фар европейских производителей в СПб — от 3 500 ₽ |…</v>
       </c>
     </row>
@@ -1635,21 +2403,45 @@
         <v>Ремонт фар</v>
       </c>
       <c r="G33" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/esD-5MJQmzWE3pRTnr1UMgEKJiU-960.jpg</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 2 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L33" t="str">
+        <v>TOYOTA|LEXUS|NISSAN|HONDA|MAZDA|MITSUBISHI|SUBARU|SUZUKI|KIA|Hyundai|INFINITI|SsangYong</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Сколько времени занимает ремонт фар китайских производителей?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O33" t="str">
         <v>ремонт фар китайских производителей</v>
       </c>
-      <c r="H33" t="str">
+      <c r="P33" t="str">
         <v>Ремонт фар китайских производителей в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="I33" t="str">
+      <c r="Q33" t="str">
         <v>Восстанавливаем фары китайских марок — часто неразборные LED-модули и нестандартная геометрия. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J33" t="str">
+      <c r="R33" t="str">
         <v>ремонт фар китайских производителей, ремонт фар китайских производителей спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K33" t="str">
+      <c r="S33" t="str">
         <v>Ремонт фар китайских производителей в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="L33" t="str">
+      <c r="T33" t="str">
         <v>Ремонт фар китайских производителей в СПб — от 2 500 ₽ | КБ…</v>
       </c>
     </row>
@@ -1673,21 +2465,45 @@
         <v>Ремонт фар</v>
       </c>
       <c r="G34" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-23.jpg</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 3 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L34" t="str">
+        <v>FORD|CHEVROLET|CADILLAC|JEEP|DODGE|CHRYSLER|HUMMER|ACURA</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Сколько времени занимает ремонт фар американского рынка?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O34" t="str">
         <v>ремонт фар американского рынка</v>
       </c>
-      <c r="H34" t="str">
+      <c r="P34" t="str">
         <v>Ремонт фар американского рынка в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I34" t="str">
+      <c r="Q34" t="str">
         <v>Ремонт оптики американского рынка — отличия в креплениях, проводке и светораспределении. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J34" t="str">
+      <c r="R34" t="str">
         <v>ремонт фар американского рынка, ремонт фар американского рынка спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K34" t="str">
+      <c r="S34" t="str">
         <v>Ремонт фар американского рынка в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L34" t="str">
+      <c r="T34" t="str">
         <v>Ремонт фар американского рынка в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1711,21 +2527,45 @@
         <v>Регулировка и диагностика</v>
       </c>
       <c r="G35" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2021/06/RagnnEphveQZgBY29n3396qgdmc-9601.jpg</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Диагностика системы AFS::Входит в стоимость::30-60 мин::-|Ремонт / адаптация AFS::от 4 000 ₽::2-6 ч::1 год</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Замена датчиков / блоков::по согласованию::+2-4 ч::по запчасти</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L35" t="str">
+        <v>BMW|MERCEDES|AUDI|LEXUS|PORSCHE|Land Rover|JAGUAR|INFINITI|Maserati|BENTLEY</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Сколько времени занимает ремонт систем адаптивного освещения?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O35" t="str">
         <v>ремонт систем адаптивного освещения</v>
       </c>
-      <c r="H35" t="str">
+      <c r="P35" t="str">
         <v>Ремонт систем адаптивного освещения (AFS) в СПб — от 4 000…</v>
       </c>
-      <c r="I35" t="str">
+      <c r="Q35" t="str">
         <v>Диагностика и ремонт AFS: моторы, датчики, блоки управления. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J35" t="str">
+      <c r="R35" t="str">
         <v>ремонт систем адаптивного освещения, ремонт систем адаптивного освещения спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K35" t="str">
+      <c r="S35" t="str">
         <v>Ремонт систем адаптивного освещения (AFS) в СПб — от 4 000…</v>
       </c>
-      <c r="L35" t="str">
+      <c r="T35" t="str">
         <v>Ремонт систем адаптивного освещения (AFS) в СПб — от 4 000…</v>
       </c>
     </row>
@@ -1749,21 +2589,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G36" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/avensis-1.jpeg</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Вакуумное напыление отражателей::от 6 000 ₽::1-2 дня::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L36" t="str">
+        <v>BMW|MERCEDES|AUDI|LEXUS|PORSCHE|Land Rover|JAGUAR|INFINITI|Maserati|BENTLEY</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Сколько времени занимает восстановление отражателей методом вакуумного напыления?::Вакуумное напыление занимает 1–2 рабочих дня.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O36" t="str">
         <v>восстановление отражателей методом вакуумного напыления</v>
       </c>
-      <c r="H36" t="str">
+      <c r="P36" t="str">
         <v>Восстановление отражателей методом вакуумного напыления в С…</v>
       </c>
-      <c r="I36" t="str">
+      <c r="Q36" t="str">
         <v>Восстанавливаем выгоревшие отражатели методом вакуумного напыления — заводское качество отражения. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J36" t="str">
+      <c r="R36" t="str">
         <v>восстановление отражателей методом вакуумного напыления, восстановление отражателей методом вакуумного напыления спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K36" t="str">
+      <c r="S36" t="str">
         <v>Восстановление отражателей методом вакуумного напыления в С…</v>
       </c>
-      <c r="L36" t="str">
+      <c r="T36" t="str">
         <v>Восстановление отражателей методом вакуумного напыления в С…</v>
       </c>
     </row>
@@ -1787,21 +2651,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G37" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-9.jpg</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт / перепайка платы::от 4 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L37" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Сколько времени занимает ремонт и перепайка драйверов?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O37" t="str">
         <v>ремонт/перепайка драйверов</v>
       </c>
-      <c r="H37" t="str">
+      <c r="P37" t="str">
         <v>Ремонт/перепайка драйверов (плат) LED в СПб — от 4 000 ₽ |…</v>
       </c>
-      <c r="I37" t="str">
+      <c r="Q37" t="str">
         <v>Перепаиваем LED-драйверы и платы управления в фарах и фонарях. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J37" t="str">
+      <c r="R37" t="str">
         <v>ремонт/перепайка драйверов, ремонт/перепайка драйверов спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K37" t="str">
+      <c r="S37" t="str">
         <v>Ремонт/перепайка драйверов (плат) LED в СПб — от 4 000 ₽ |…</v>
       </c>
-      <c r="L37" t="str">
+      <c r="T37" t="str">
         <v>Ремонт/перепайка драйверов (плат) LED в СПб — от 4 000 ₽ |…</v>
       </c>
     </row>
@@ -1825,21 +2713,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G38" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/harness.jpeg</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт / перепайка платы::от 5 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L38" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M38" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Сколько времени занимает ремонт контроллеров управления фарой?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O38" t="str">
         <v>ремонт контроллеров управления фарой</v>
       </c>
-      <c r="H38" t="str">
+      <c r="P38" t="str">
         <v>Ремонт контроллеров управления фарой (ЭБУ) в СПб — от 5 000…</v>
       </c>
-      <c r="I38" t="str">
+      <c r="Q38" t="str">
         <v>Ремонт и прошивка блоков управления фарой. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J38" t="str">
+      <c r="R38" t="str">
         <v>ремонт контроллеров управления фарой, ремонт контроллеров управления фарой спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K38" t="str">
+      <c r="S38" t="str">
         <v>Ремонт контроллеров управления фарой (ЭБУ) в СПб — от 5 000…</v>
       </c>
-      <c r="L38" t="str">
+      <c r="T38" t="str">
         <v>Ремонт контроллеров управления фарой (ЭБУ) в СПб — от 5 000…</v>
       </c>
     </row>
@@ -1863,21 +2775,45 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G39" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/nwAAAgARPOA-19201.jpg</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Химическая чистка изнутри::от 2 500 ₽::2-3 ч::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L39" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Сколько времени занимает химическая чистка фары изнутри?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O39" t="str">
         <v>химчистка фары изнутри</v>
       </c>
-      <c r="H39" t="str">
+      <c r="P39" t="str">
         <v>Химчистка фары изнутри в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I39" t="str">
+      <c r="Q39" t="str">
         <v>Удаляем налёт и помутнение изнутри фары без разборки корпуса. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J39" t="str">
+      <c r="R39" t="str">
         <v>химчистка фары изнутри, химчистка фары изнутри спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K39" t="str">
+      <c r="S39" t="str">
         <v>Химчистка фары изнутри в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L39" t="str">
+      <c r="T39" t="str">
         <v>Химчистка фары изнутри в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1901,21 +2837,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G40" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/2013-dodge-ram-1500-quad-laramie-truck-angular-front.png</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Компьютерная диагностика::Входит в стоимость::30 мин::-|Кодирование / программирование::от 2 000 ₽::1-2 ч::-</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Установка «обманок» (при необходимости)::от 1 500 ₽::+30 мин::1 год</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L40" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Сколько времени занимает программное отключение опроса ламп?::Диагностика и кодирование — обычно 1–2 часа.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
+      </c>
+      <c r="O40" t="str">
         <v>программное отключение опроса ламп</v>
       </c>
-      <c r="H40" t="str">
+      <c r="P40" t="str">
         <v>Программное отключение опроса ламп («обманки») в СПб — от 2…</v>
       </c>
-      <c r="I40" t="str">
+      <c r="Q40" t="str">
         <v>Кодируем ЭБУ или ставим обманки — без ошибок на панели. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J40" t="str">
+      <c r="R40" t="str">
         <v>программное отключение опроса ламп, программное отключение опроса ламп спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K40" t="str">
+      <c r="S40" t="str">
         <v>Программное отключение опроса ламп («обманки») в СПб — от 2…</v>
       </c>
-      <c r="L40" t="str">
+      <c r="T40" t="str">
         <v>Программное отключение опроса ламп («обманки») в СПб — от 2…</v>
       </c>
     </row>
@@ -1939,21 +2899,45 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G41" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/sT1Au9E5E4tZRh3x-yY-TtGRJck-1920.jpg</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 2 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L41" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N41" t="str">
+        <v>Сколько времени занимает замена внутренней проводки фары?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O41" t="str">
         <v>замена внутренней проводки фары</v>
       </c>
-      <c r="H41" t="str">
+      <c r="P41" t="str">
         <v>Замена внутренней проводки фары в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="I41" t="str">
+      <c r="Q41" t="str">
         <v>Меняем перегоревшую или повреждённую проводку внутри фары. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J41" t="str">
+      <c r="R41" t="str">
         <v>замена внутренней проводки фары, замена внутренней проводки фары спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K41" t="str">
+      <c r="S41" t="str">
         <v>Замена внутренней проводки фары в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="L41" t="str">
+      <c r="T41" t="str">
         <v>Замена внутренней проводки фары в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1977,21 +2961,45 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G42" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/hoAAAgDOIuA-19201.jpg</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Установка автокорректора::от 4 000 ₽::2-4 ч::1 год|Калибровка светового пучка::входит в стоимость::30 мин::-</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Адаптация / кодирование::от 2 000 ₽::+1 ч::-</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L42" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N42" t="str">
+        <v>Сколько времени занимает установка автокорректоров фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
+      </c>
+      <c r="O42" t="str">
         <v>установка автокорректоров фар</v>
       </c>
-      <c r="H42" t="str">
+      <c r="P42" t="str">
         <v>Установка автокорректоров фар в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="I42" t="str">
+      <c r="Q42" t="str">
         <v>Монтируем автокорректоры с подключением к штатной системе. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J42" t="str">
+      <c r="R42" t="str">
         <v>установка автокорректоров фар, установка автокорректоров фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K42" t="str">
+      <c r="S42" t="str">
         <v>Установка автокорректоров фар в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="L42" t="str">
+      <c r="T42" t="str">
         <v>Установка автокорректоров фар в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2015,27 +3023,51 @@
         <v>Регулировка и диагностика</v>
       </c>
       <c r="G43" t="str">
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/heads.png</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Компьютерная диагностика::Входит в стоимость::30 мин::-|Кодирование / программирование::от 3 000 ₽::1-2 ч::-</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Установка «обманок» (при необходимости)::от 1 500 ₽::+30 мин::1 год</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="L43" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="N43" t="str">
+        <v>Сколько времени занимает кодирование и программирование штатных блоков управления светом + компьютерная диагностика?::Диагностика и кодирование — обычно 1–2 часа.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
+      </c>
+      <c r="O43" t="str">
         <v>кодирование/программирование блоков + диагностика</v>
       </c>
-      <c r="H43" t="str">
+      <c r="P43" t="str">
         <v>Кодирование/программирование блоков + диагностика в СПб — о…</v>
       </c>
-      <c r="I43" t="str">
+      <c r="Q43" t="str">
         <v>Кодируем блоки света, активируем функции, проводим компьютерную диагностику. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="J43" t="str">
+      <c r="R43" t="str">
         <v>кодирование/программирование блоков + диагностика, кодирование/программирование блоков + диагностика спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="K43" t="str">
+      <c r="S43" t="str">
         <v>Кодирование/программирование блоков + диагностика в СПб — о…</v>
       </c>
-      <c r="L43" t="str">
+      <c r="T43" t="str">
         <v>Кодирование/программирование блоков + диагностика в СПб — о…</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update single service block
</commit_message>
<xml_diff>
--- a/parsing/data/services-import.xlsx
+++ b/parsing/data/services-import.xlsx
@@ -481,7 +481,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G2" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/biled.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/e84.jpg</v>
       </c>
       <c r="H2" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 8 500 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -543,7 +543,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G3" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/YYAAAgDI0OA-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2023/03/A0uDlazmT8Im_nUrRIfPLQVxYZs-960.jpg</v>
       </c>
       <c r="H3" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка лазерных модулей::от 35 000 ₽ / шт.::3-5 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -667,7 +667,7 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G5" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/8FeX41yZ3b2mVdd1jWi45NW5uoY-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/e90.jpg</v>
       </c>
       <c r="H5" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 2 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -853,7 +853,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G8" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-36.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/biled.jpg</v>
       </c>
       <c r="H8" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 8 500 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -977,7 +977,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G10" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/09/F4AAAgKEmOA-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/nCAAAgMzVeA-19201-1.jpg</v>
       </c>
       <c r="H10" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 6 000 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -1039,7 +1039,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G11" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/5141ad6393277.jpeg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/2SAAAgFshOA-19201.jpg</v>
       </c>
       <c r="H11" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 2 500 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -1163,7 +1163,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G13" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/kyaaagkceoa-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/08/IMG_4529.jpg</v>
       </c>
       <c r="H13" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 5 000 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -1473,7 +1473,7 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G18" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/06/YoAAAgFugOA-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/f01led.jpg</v>
       </c>
       <c r="H18" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт светодиодных модулей::от 4 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -1535,7 +1535,7 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G19" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/rear-1.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-9.jpg</v>
       </c>
       <c r="H19" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт светодиодных модулей::от 3 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -1597,7 +1597,7 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G20" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/ledfog.png</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/6f637804k444-19201.jpg</v>
       </c>
       <c r="H20" t="str">
         <v>Установка ПТФ::от 6 000 ₽::2-4 ч::1 год|Программная активация (при необходимости)::входит в стоимость / от 2 000 ₽::+30-60 мин::-</v>
@@ -1659,7 +1659,7 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G21" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-35.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/EAAAAgNVReA-19201.jpg</v>
       </c>
       <c r="H21" t="str">
         <v>Установка ПТФ::от 5 000 ₽::2-4 ч::1 год|Программная активация (при необходимости)::входит в стоимость / от 2 000 ₽::+30-60 мин::-</v>
@@ -1721,7 +1721,7 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G22" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/07/s0AAAgHi0OA-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/i-AAAgO2yeA-9601.jpg</v>
       </c>
       <c r="H22" t="str">
         <v>Замена стёкол ПТФ::от 3 000 ₽::30-90 мин::6 мес.</v>
@@ -1783,7 +1783,7 @@
         <v>Противотуманные фары (ПТФ)</v>
       </c>
       <c r="G23" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-8.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/6f637804k444-19201.jpg</v>
       </c>
       <c r="H23" t="str">
         <v>Замена ламп в ПТФ::от 1 500 ₽::30-90 мин::-</v>
@@ -1845,7 +1845,7 @@
         <v>Доп. услуги</v>
       </c>
       <c r="G24" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/08/img_3959.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/e53.jpg</v>
       </c>
       <c r="H24" t="str">
         <v>Замена ламп на светодиодные::от 2 000 ₽::30-90 мин::1 год</v>
@@ -1907,7 +1907,7 @@
         <v>Механика</v>
       </c>
       <c r="G25" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/e-repair-1.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/sequoia-1.jpg</v>
       </c>
       <c r="H25" t="str">
         <v>Диагностика узла::Входит в стоимость::30 мин::-|Ремонт механики::от 2 500 ₽::1-3 ч::1 год</v>
@@ -1969,7 +1969,7 @@
         <v>Механика</v>
       </c>
       <c r="G26" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/how-to-choose-the-best-car-amplifier.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/08/IMG_toyota-nolden-pioneer-bixenon-1.jpg</v>
       </c>
       <c r="H26" t="str">
         <v>Диагностика узла::Входит в стоимость::30 мин::-|Ремонт механики::от 2 000 ₽::1-3 ч::1 год</v>
@@ -2155,7 +2155,7 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G29" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/syAAAgDNyeA-19201.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/h0AAAgEVyeA-9601.jpg</v>
       </c>
       <c r="H29" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Восстановление креплений («ушек»)::от 2 500 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2217,7 +2217,7 @@
         <v>Механика</v>
       </c>
       <c r="G30" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/6f836g4k337-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/m37-1.jpg</v>
       </c>
       <c r="H30" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 3 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2279,7 +2279,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G31" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/QwisvkNREXiXiDRRslmWElJGht4-960.jpg</v>
+        <v>https://ksenonspb.ru/portfolio/7MAAAgAzWOA-1920.jpg</v>
       </c>
       <c r="H31" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 5 000 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2341,7 +2341,7 @@
         <v>Ремонт фар</v>
       </c>
       <c r="G32" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2022/04/S7jUlvfRpkxQN06kpudCI9as0o-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/16c6149s-960.jpg</v>
       </c>
       <c r="H32" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 3 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2403,7 +2403,7 @@
         <v>Ремонт фар</v>
       </c>
       <c r="G33" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/esD-5MJQmzWE3pRTnr1UMgEKJiU-960.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/11/KFAAAgLSoeA-9601.jpg</v>
       </c>
       <c r="H33" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 2 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2465,7 +2465,7 @@
         <v>Ремонт фар</v>
       </c>
       <c r="G34" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-23.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/BYAAAgOQwuA-19201.jpg</v>
       </c>
       <c r="H34" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 3 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2527,7 +2527,7 @@
         <v>Регулировка и диагностика</v>
       </c>
       <c r="G35" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2021/06/RagnnEphveQZgBY29n3396qgdmc-9601.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/b6ceb9ds-960.jpg</v>
       </c>
       <c r="H35" t="str">
         <v>Диагностика системы AFS::Входит в стоимость::30-60 мин::-|Ремонт / адаптация AFS::от 4 000 ₽::2-6 ч::1 год</v>
@@ -2589,7 +2589,7 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G36" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/avensis-1.jpeg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/reflector-1.png</v>
       </c>
       <c r="H36" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Вакуумное напыление отражателей::от 6 000 ₽::1-2 дня::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2651,7 +2651,7 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G37" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-9.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/SGAAAgIfOeA-19201.jpg</v>
       </c>
       <c r="H37" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт / перепайка платы::от 4 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2713,7 +2713,7 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G38" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/harness.jpeg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/e-repair-1.jpg</v>
       </c>
       <c r="H38" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт / перепайка платы::от 5 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2775,7 +2775,7 @@
         <v>Оптика и корпус</v>
       </c>
       <c r="G39" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/nwAAAgARPOA-19201.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/cleaning-1.jpg</v>
       </c>
       <c r="H39" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Химическая чистка изнутри::от 2 500 ₽::2-3 ч::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2837,7 +2837,7 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G40" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/2013-dodge-ram-1500-quad-laramie-truck-angular-front.png</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-23.jpg</v>
       </c>
       <c r="H40" t="str">
         <v>Компьютерная диагностика::Входит в стоимость::30 мин::-|Кодирование / программирование::от 2 000 ₽::1-2 ч::-</v>
@@ -2899,7 +2899,7 @@
         <v>Электрика и электроника</v>
       </c>
       <c r="G41" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2026/01/sT1Au9E5E4tZRh3x-yY-TtGRJck-1920.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2021/09/5D7ZL-EXgUe6NbclWgUam9SMyS0-9601.jpg</v>
       </c>
       <c r="H41" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 2 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
@@ -2961,7 +2961,7 @@
         <v>Тюнинг фар</v>
       </c>
       <c r="G42" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2020/03/hoAAAgDOIuA-19201.jpg</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2021/09/IKgT7yLzjx-1W7XenovHwM91Iys-960.jpg</v>
       </c>
       <c r="H42" t="str">
         <v>Установка автокорректора::от 4 000 ₽::2-4 ч::1 год|Калибровка светового пучка::входит в стоимость::30 мин::-</v>
@@ -3023,7 +3023,7 @@
         <v>Регулировка и диагностика</v>
       </c>
       <c r="G43" t="str">
-        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/heads.png</v>
+        <v>https://ksenonspb.ru/wp-content/uploads/2016/09/e-repair-1.jpg</v>
       </c>
       <c r="H43" t="str">
         <v>Компьютерная диагностика::Входит в стоимость::30 мин::-|Кодирование / программирование::от 3 000 ₽::1-2 ч::-</v>

</xml_diff>

<commit_message>
feat: add pricing page
</commit_message>
<xml_diff>
--- a/parsing/data/services-import.xlsx
+++ b/parsing/data/services-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T43"/>
+  <dimension ref="A1:V43"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,54 +410,60 @@
         <v>price</v>
       </c>
       <c r="D1" t="str">
+        <v>duration</v>
+      </c>
+      <c r="E1" t="str">
+        <v>price_note</v>
+      </c>
+      <c r="F1" t="str">
         <v>desc</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>benefits</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>category</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>image</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>price_main</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>price_extra</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>price_diagnostics</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>warranty_text</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>related_brands</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>faq_title</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>faq</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>Focus Keyword</v>
       </c>
-      <c r="P1" t="str">
+      <c r="R1" t="str">
         <v>SEO Title</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>Meta Description</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>Meta Keywords</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>Facebook Title</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Twitter Title</v>
       </c>
     </row>
@@ -472,54 +478,60 @@
         <v>8500</v>
       </c>
       <c r="D2" t="str">
+        <v>2-3 ч</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>Меняем выгоревшие линзы на модули Xenon или Bi-LED.</v>
       </c>
-      <c r="E2" t="str">
+      <c r="G2" t="str">
         <v>Гарантия 2 года на модули</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/e84.jpg</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 8 500 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J2" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L2" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M2" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N2" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P2" t="str">
         <v>Сколько времени занимает замена линз в фарах?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 8 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O2" t="str">
+      <c r="Q2" t="str">
         <v>установка линз</v>
       </c>
-      <c r="P2" t="str">
+      <c r="R2" t="str">
         <v>Установка линз (Xenon/Bi-LED) в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="S2" t="str">
         <v>Меняем выгоревшие линзы на модули Xenon или Bi-LED. Цена от 8 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R2" t="str">
+      <c r="T2" t="str">
         <v>установка линз, установка линз спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S2" t="str">
+      <c r="U2" t="str">
         <v>Установка линз (Xenon/Bi-LED) в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T2" t="str">
+      <c r="V2" t="str">
         <v>Установка линз (Xenon/Bi-LED) в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -534,54 +546,60 @@
         <v>35000</v>
       </c>
       <c r="D3" t="str">
+        <v>3-5 ч</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>Топовые лазерные модули с дальним светом до 600 м. Для тех, кто хочет максимум.</v>
       </c>
-      <c r="E3" t="str">
+      <c r="G3" t="str">
         <v>Дальний свет в 3+ ярче штатного</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2023/03/A0uDlazmT8Im_nUrRIfPLQVxYZs-960.jpg</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка лазерных модулей::от 35 000 ₽ / шт.::3-5 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J3" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L3" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="N3" t="str">
         <v>BMW|MERCEDES|AUDI|LEXUS|PORSCHE|Land Rover|JAGUAR|INFINITI|Maserati|BENTLEY</v>
       </c>
-      <c r="M3" t="str">
-        <v>Частые вопросы</v>
-      </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P3" t="str">
         <v>Сколько времени занимает установка лазерных?::Установка лазерных модулей — обычно 3–5 часов.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 35 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O3" t="str">
+      <c r="Q3" t="str">
         <v>установка лазерных</v>
       </c>
-      <c r="P3" t="str">
+      <c r="R3" t="str">
         <v>Установка лазерных (Laser) линз в СПб — от 35 000 ₽ | КБ АВ…</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="S3" t="str">
         <v>Топовые лазерные модули с дальним светом до 600 м. Для тех, кто хочет максимум. Цена от 35 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>установка лазерных, установка лазерных спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
         <v>Установка лазерных (Laser) линз в СПб — от 35 000 ₽ | КБ АВ…</v>
       </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
         <v>Установка лазерных (Laser) линз в СПб — от 35 000 ₽ | КБ АВ…</v>
       </c>
     </row>
@@ -596,54 +614,60 @@
         <v>2500</v>
       </c>
       <c r="D4" t="str">
+        <v>1-2 ч</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>Глубокая шлифовка и полировка — возвращаем прозрачность без замены стекла.</v>
       </c>
-      <c r="E4" t="str">
+      <c r="G4" t="str">
         <v>Как новые, Без замены стекла</v>
       </c>
-      <c r="F4" t="str">
+      <c r="H4" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/polish-1.jpg</v>
       </c>
-      <c r="H4" t="str">
+      <c r="J4" t="str">
         <v>Шлифовка и полировка стекла::от 2 500 ₽::1-2 ч::6 мес.|Защитное покрытие::входит в стоимость::30 мин::-</v>
       </c>
-      <c r="I4" t="str">
+      <c r="K4" t="str">
         <v>Полировка изнутри (при разборке)::от 1 500 ₽::+1 ч::1 год|Устранение глубоких царапин::от 1 000 ₽::+1 ч::-</v>
       </c>
-      <c r="J4" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L4" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M4" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N4" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P4" t="str">
         <v>Сколько времени занимает полировка и шлифовка фар?::Обычно 1–2 часа на пару фар.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O4" t="str">
+      <c r="Q4" t="str">
         <v>полировка и шлифовка фар</v>
       </c>
-      <c r="P4" t="str">
+      <c r="R4" t="str">
         <v>Полировка и шлифовка фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="S4" t="str">
         <v>Глубокая шлифовка и полировка — возвращаем прозрачность без замены стекла. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R4" t="str">
+      <c r="T4" t="str">
         <v>полировка и шлифовка фар, полировка и шлифовка фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S4" t="str">
+      <c r="U4" t="str">
         <v>Полировка и шлифовка фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T4" t="str">
+      <c r="V4" t="str">
         <v>Полировка и шлифовка фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -658,54 +682,60 @@
         <v>2500</v>
       </c>
       <c r="D5" t="str">
+        <v>от 2 ч</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>Восстанавливаем фары после ДТП, заливов и выгорания LED. От галогена до лазерных модулей.</v>
       </c>
-      <c r="E5" t="str">
+      <c r="G5" t="str">
         <v>Дешевле замены в 5-10 раз</v>
       </c>
-      <c r="F5" t="str">
+      <c r="H5" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G5" t="str">
+      <c r="I5" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/e90.jpg</v>
       </c>
-      <c r="H5" t="str">
+      <c r="J5" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 2 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I5" t="str">
+      <c r="K5" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J5" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L5" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M5" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N5" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P5" t="str">
         <v>Сколько времени занимает ремонт фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O5" t="str">
+      <c r="Q5" t="str">
         <v>ремонт фар</v>
       </c>
-      <c r="P5" t="str">
+      <c r="R5" t="str">
         <v>Ремонт фар (комплексный) в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="S5" t="str">
         <v>Восстанавливаем фары после ДТП, заливов и выгорания LED. От галогена до лазерных модулей. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R5" t="str">
+      <c r="T5" t="str">
         <v>ремонт фар, ремонт фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S5" t="str">
+      <c r="U5" t="str">
         <v>Ремонт фар (комплексный) в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T5" t="str">
+      <c r="V5" t="str">
         <v>Ремонт фар (комплексный) в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -720,54 +750,60 @@
         <v>5000</v>
       </c>
       <c r="D6" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
         <v>Демонтируем треснувшее или мутное стекло, устанавливаем новое с герметизацией корпуса.</v>
       </c>
-      <c r="E6" t="str">
+      <c r="G6" t="str">
         <v>Не запотеет</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G6" t="str">
+      <c r="I6" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/08/img_6069.jpg</v>
       </c>
-      <c r="H6" t="str">
+      <c r="J6" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена стекла фары::от 5 000 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I6" t="str">
+      <c r="K6" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J6" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L6" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M6" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N6" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P6" t="str">
         <v>Сколько времени занимает замена стёкол фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O6" t="str">
+      <c r="Q6" t="str">
         <v>замена стёкол фар</v>
       </c>
-      <c r="P6" t="str">
+      <c r="R6" t="str">
         <v>Замена стёкол фар в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="S6" t="str">
         <v>Демонтируем треснувшее или мутное стекло, устанавливаем новое с герметизацией корпуса. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R6" t="str">
+      <c r="T6" t="str">
         <v>замена стёкол фар, замена стёкол фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S6" t="str">
+      <c r="U6" t="str">
         <v>Замена стёкол фар в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T6" t="str">
+      <c r="V6" t="str">
         <v>Замена стёкол фар в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -782,54 +818,60 @@
         <v>3500</v>
       </c>
       <c r="D7" t="str">
+        <v>2-3 ч</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
         <v>Диагностируем причину, переклеиваем корпус по заводским технологиям.</v>
       </c>
-      <c r="E7" t="str">
+      <c r="G7" t="str">
         <v>Гарантия от запотевания 1 год</v>
       </c>
-      <c r="F7" t="str">
+      <c r="H7" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G7" t="str">
+      <c r="I7" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/misted-1.jpg</v>
       </c>
-      <c r="H7" t="str">
+      <c r="J7" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Устранение запотевания и просушка::от 3 500 ₽::2-3 ч::1 год|Замена уплотнителя / клапанов::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I7" t="str">
+      <c r="K7" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J7" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L7" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M7" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N7" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P7" t="str">
         <v>Сколько времени занимает устранение запотевания фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O7" t="str">
+      <c r="Q7" t="str">
         <v>устранение запотевания фар</v>
       </c>
-      <c r="P7" t="str">
+      <c r="R7" t="str">
         <v>Устранение запотевания фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q7" t="str">
+      <c r="S7" t="str">
         <v>Диагностируем причину, переклеиваем корпус по заводским технологиям. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R7" t="str">
+      <c r="T7" t="str">
         <v>устранение запотевания фар, устранение запотевания фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S7" t="str">
+      <c r="U7" t="str">
         <v>Устранение запотевания фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T7" t="str">
+      <c r="V7" t="str">
         <v>Устранение запотевания фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -844,54 +886,60 @@
         <v>8500</v>
       </c>
       <c r="D8" t="str">
+        <v>2-3 ч</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
         <v>Переходим на качественный диодный свет. Ярче ксенона, без слепящего встречного потока.</v>
       </c>
-      <c r="E8" t="str">
+      <c r="G8" t="str">
         <v>Срок службы до 50 000 ч</v>
       </c>
-      <c r="F8" t="str">
+      <c r="H8" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G8" t="str">
+      <c r="I8" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/biled.jpg</v>
       </c>
-      <c r="H8" t="str">
+      <c r="J8" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 8 500 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I8" t="str">
+      <c r="K8" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J8" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L8" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M8" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N8" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P8" t="str">
         <v>Сколько времени занимает установка bi-led?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 8 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O8" t="str">
+      <c r="Q8" t="str">
         <v>установка bi-led линз</v>
       </c>
-      <c r="P8" t="str">
+      <c r="R8" t="str">
         <v>Установка Bi-LED линз в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="S8" t="str">
         <v>Переходим на качественный диодный свет. Ярче ксенона, без слепящего встречного потока. Цена от 8 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R8" t="str">
+      <c r="T8" t="str">
         <v>установка bi-led линз, установка bi-led линз спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S8" t="str">
+      <c r="U8" t="str">
         <v>Установка Bi-LED линз в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T8" t="str">
+      <c r="V8" t="str">
         <v>Установка Bi-LED линз в СПб — от 8 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -906,54 +954,60 @@
         <v>5000</v>
       </c>
       <c r="D9" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>Монтируем штатные ксеноновые комплекты с правильной фокусировкой и герметизацией.</v>
       </c>
-      <c r="E9" t="str">
+      <c r="G9" t="str">
         <v>Штатное решение, Гарантия</v>
       </c>
-      <c r="F9" t="str">
+      <c r="H9" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G9" t="str">
+      <c r="I9" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/xenon.jpg</v>
       </c>
-      <c r="H9" t="str">
+      <c r="J9" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка ксенонового комплекта::от 5 000 ₽::2-4 ч::1 год|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I9" t="str">
+      <c r="K9" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J9" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K9" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L9" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M9" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N9" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P9" t="str">
         <v>Сколько времени занимает установка ксенона?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O9" t="str">
+      <c r="Q9" t="str">
         <v>установка ксенона</v>
       </c>
-      <c r="P9" t="str">
+      <c r="R9" t="str">
         <v>Установка ксенона (штатные комплекты) в СПб — от 5 000 ₽ |…</v>
       </c>
-      <c r="Q9" t="str">
+      <c r="S9" t="str">
         <v>Монтируем штатные ксеноновые комплекты с правильной фокусировкой и герметизацией. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R9" t="str">
+      <c r="T9" t="str">
         <v>установка ксенона, установка ксенона спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S9" t="str">
+      <c r="U9" t="str">
         <v>Установка ксенона (штатные комплекты) в СПб — от 5 000 ₽ |…</v>
       </c>
-      <c r="T9" t="str">
+      <c r="V9" t="str">
         <v>Установка ксенона (штатные комплекты) в СПб — от 5 000 ₽ |…</v>
       </c>
     </row>
@@ -968,54 +1022,60 @@
         <v>6000</v>
       </c>
       <c r="D10" t="str">
+        <v>2-3 ч</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
         <v>Меняем заводские линзы на оригинал или проверенный аналог с настройкой света.</v>
       </c>
-      <c r="E10" t="str">
+      <c r="G10" t="str">
         <v>Оригинал или аналог</v>
       </c>
-      <c r="F10" t="str">
+      <c r="H10" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G10" t="str">
+      <c r="I10" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/nCAAAgMzVeA-19201-1.jpg</v>
       </c>
-      <c r="H10" t="str">
+      <c r="J10" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 6 000 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I10" t="str">
+      <c r="K10" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J10" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K10" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L10" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M10" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N10" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P10" t="str">
         <v>Сколько времени занимает замена штатных линз на оригинал или аналог?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O10" t="str">
+      <c r="Q10" t="str">
         <v>замена штатных линз на оригинал/аналог</v>
       </c>
-      <c r="P10" t="str">
+      <c r="R10" t="str">
         <v>Замена штатных линз на оригинал/аналог в СПб — от 6 000 ₽ |…</v>
       </c>
-      <c r="Q10" t="str">
+      <c r="S10" t="str">
         <v>Меняем заводские линзы на оригинал или проверенный аналог с настройкой света. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R10" t="str">
+      <c r="T10" t="str">
         <v>замена штатных линз на оригинал/аналог, замена штатных линз на оригинал/аналог спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S10" t="str">
+      <c r="U10" t="str">
         <v>Замена штатных линз на оригинал/аналог в СПб — от 6 000 ₽ |…</v>
       </c>
-      <c r="T10" t="str">
+      <c r="V10" t="str">
         <v>Замена штатных линз на оригинал/аналог в СПб — от 6 000 ₽ |…</v>
       </c>
     </row>
@@ -1030,54 +1090,60 @@
         <v>2500</v>
       </c>
       <c r="D11" t="str">
+        <v>3-8 ч</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
         <v>Устанавливаем ангельские и дьявольские глазки с аккуратной проводкой и герметизацией.</v>
       </c>
-      <c r="E11" t="str">
+      <c r="G11" t="str">
         <v>Индивидуальный дизайн</v>
       </c>
-      <c r="F11" t="str">
+      <c r="H11" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G11" t="str">
+      <c r="I11" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/2SAAAgFshOA-19201.jpg</v>
       </c>
-      <c r="H11" t="str">
+      <c r="J11" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 2 500 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I11" t="str">
+      <c r="K11" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J11" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K11" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L11" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M11" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N11" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P11" t="str">
         <v>Сколько времени занимает тюнинг подсветки?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O11" t="str">
+      <c r="Q11" t="str">
         <v>тюнинг подсветки</v>
       </c>
-      <c r="P11" t="str">
+      <c r="R11" t="str">
         <v>Тюнинг подсветки (Ангельские/Дьявольские глазки) в СПб — от…</v>
       </c>
-      <c r="Q11" t="str">
+      <c r="S11" t="str">
         <v>Устанавливаем ангельские и дьявольские глазки с аккуратной проводкой и герметизацией. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R11" t="str">
+      <c r="T11" t="str">
         <v>тюнинг подсветки, тюнинг подсветки спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S11" t="str">
+      <c r="U11" t="str">
         <v>Тюнинг подсветки (Ангельские/Дьявольские глазки) в СПб — от…</v>
       </c>
-      <c r="T11" t="str">
+      <c r="V11" t="str">
         <v>Тюнинг подсветки (Ангельские/Дьявольские глазки) в СПб — от…</v>
       </c>
     </row>
@@ -1092,54 +1158,60 @@
         <v>3500</v>
       </c>
       <c r="D12" t="str">
+        <v>1 день</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
         <v>Красим внутренние маски термостойкой краской — чёрный, хром или под ваш стиль.</v>
       </c>
-      <c r="E12" t="str">
+      <c r="G12" t="str">
         <v>Термостойкая краска</v>
       </c>
-      <c r="F12" t="str">
+      <c r="H12" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G12" t="str">
+      <c r="I12" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/paint.png</v>
       </c>
-      <c r="H12" t="str">
+      <c r="J12" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Покраска масок фар::от 3 500 ₽::1 день::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I12" t="str">
+      <c r="K12" t="str">
         <v>Покраска декоративных элементов::от 1 500 ₽::+4 ч::-|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J12" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K12" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L12" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M12" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N12" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P12" t="str">
         <v>Сколько времени занимает покраска масок фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O12" t="str">
+      <c r="Q12" t="str">
         <v>покраска масок фар</v>
       </c>
-      <c r="P12" t="str">
+      <c r="R12" t="str">
         <v>Покраска масок фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q12" t="str">
+      <c r="S12" t="str">
         <v>Красим внутренние маски термостойкой краской — чёрный, хром или под ваш стиль. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R12" t="str">
+      <c r="T12" t="str">
         <v>покраска масок фар, покраска масок фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S12" t="str">
+      <c r="U12" t="str">
         <v>Покраска масок фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T12" t="str">
+      <c r="V12" t="str">
         <v>Покраска масок фар в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1154,54 +1226,60 @@
         <v>5000</v>
       </c>
       <c r="D13" t="str">
+        <v>3-8 ч</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
         <v>Делаем индивидуальные ДХО под вашу оптику с заводской герметичностью.</v>
       </c>
-      <c r="E13" t="str">
+      <c r="G13" t="str">
         <v>Индивидуальное решение</v>
       </c>
-      <c r="F13" t="str">
+      <c r="H13" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G13" t="str">
+      <c r="I13" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/08/IMG_4529.jpg</v>
       </c>
-      <c r="H13" t="str">
+      <c r="J13" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 5 000 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I13" t="str">
+      <c r="K13" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J13" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K13" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L13" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M13" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N13" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P13" t="str">
         <v>Сколько времени занимает изготовление дневных ходовых огней?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O13" t="str">
+      <c r="Q13" t="str">
         <v>изготовление дхо</v>
       </c>
-      <c r="P13" t="str">
+      <c r="R13" t="str">
         <v>Изготовление ДХО в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q13" t="str">
+      <c r="S13" t="str">
         <v>Делаем индивидуальные ДХО под вашу оптику с заводской герметичностью. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R13" t="str">
+      <c r="T13" t="str">
         <v>изготовление дхо, изготовление дхо спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S13" t="str">
+      <c r="U13" t="str">
         <v>Изготовление ДХО в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T13" t="str">
+      <c r="V13" t="str">
         <v>Изготовление ДХО в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1216,54 +1294,60 @@
         <v>2000</v>
       </c>
       <c r="D14" t="str">
+        <v>30-60 мин</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
         <v>Выставляем правильный световой пучок на стенде — без слепящего встречного.</v>
       </c>
-      <c r="E14" t="str">
+      <c r="G14" t="str">
         <v>По ГОСТ, Без слепления</v>
       </c>
-      <c r="F14" t="str">
+      <c r="H14" t="str">
         <v>Регулировка и диагностика</v>
       </c>
-      <c r="G14" t="str">
+      <c r="I14" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/reg.jpg</v>
       </c>
-      <c r="H14" t="str">
+      <c r="J14" t="str">
         <v>Регулировка на оптическом стенде::от 2 000 ₽::30-60 мин::-</v>
       </c>
-      <c r="I14" t="str">
+      <c r="K14" t="str">
         <v>Диагностика оптики перед регулировкой::Бесплатно::+15 мин::-</v>
       </c>
-      <c r="J14" t="str">
+      <c r="L14" t="str">
         <v>Проверка светового пучка::Входит в стоимость::15 мин::-</v>
       </c>
-      <c r="K14" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
-      <c r="L14" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
-      </c>
       <c r="M14" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N14" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P14" t="str">
         <v>Сколько времени занимает регулировка света фар на оптическом стенде?::Регулировка занимает 30–60 минут.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
       </c>
-      <c r="O14" t="str">
+      <c r="Q14" t="str">
         <v>регулировка света на стенде</v>
       </c>
-      <c r="P14" t="str">
+      <c r="R14" t="str">
         <v>Регулировка света на стенде в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q14" t="str">
+      <c r="S14" t="str">
         <v>Выставляем правильный световой пучок на стенде — без слепящего встречного. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R14" t="str">
+      <c r="T14" t="str">
         <v>регулировка света на стенде, регулировка света на стенде спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S14" t="str">
+      <c r="U14" t="str">
         <v>Регулировка света на стенде в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T14" t="str">
+      <c r="V14" t="str">
         <v>Регулировка света на стенде в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1278,54 +1362,60 @@
         <v>2500</v>
       </c>
       <c r="D15" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
         <v>Меняем блоки розжига и лампы, проверяем всю цепь ксенона.</v>
       </c>
-      <c r="E15" t="str">
+      <c r="G15" t="str">
         <v>Диагностика в подарок</v>
       </c>
-      <c r="F15" t="str">
+      <c r="H15" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G15" t="str">
+      <c r="I15" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/aeecc8es-960-1.jpg</v>
       </c>
-      <c r="H15" t="str">
+      <c r="J15" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 2 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I15" t="str">
+      <c r="K15" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J15" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K15" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L15" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M15" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N15" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P15" t="str">
         <v>Сколько времени занимает замена штатных блоков розжига и ламп?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O15" t="str">
+      <c r="Q15" t="str">
         <v>замена блоков розжига и ламп</v>
       </c>
-      <c r="P15" t="str">
+      <c r="R15" t="str">
         <v>Замена блоков розжига и ламп в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q15" t="str">
+      <c r="S15" t="str">
         <v>Меняем блоки розжига и лампы, проверяем всю цепь ксенона. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R15" t="str">
+      <c r="T15" t="str">
         <v>замена блоков розжига и ламп, замена блоков розжига и ламп спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S15" t="str">
+      <c r="U15" t="str">
         <v>Замена блоков розжига и ламп в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T15" t="str">
+      <c r="V15" t="str">
         <v>Замена блоков розжига и ламп в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1340,54 +1430,60 @@
         <v>3000</v>
       </c>
       <c r="D16" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
         <v>Компонентно восстанавливаем штатные дневные ходовые огни.</v>
       </c>
-      <c r="E16" t="str">
+      <c r="G16" t="str">
         <v>Штатный вид</v>
       </c>
-      <c r="F16" t="str">
+      <c r="H16" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G16" t="str">
+      <c r="I16" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/11/drQAAgC09-A-9601.jpg</v>
       </c>
-      <c r="H16" t="str">
+      <c r="J16" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 3 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I16" t="str">
+      <c r="K16" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J16" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K16" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L16" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M16" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N16" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P16" t="str">
         <v>Сколько времени занимает ремонт штатных дхо?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O16" t="str">
+      <c r="Q16" t="str">
         <v>ремонт штатных дхо</v>
       </c>
-      <c r="P16" t="str">
+      <c r="R16" t="str">
         <v>Ремонт штатных ДХО в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q16" t="str">
+      <c r="S16" t="str">
         <v>Компонентно восстанавливаем штатные дневные ходовые огни. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R16" t="str">
+      <c r="T16" t="str">
         <v>ремонт штатных дхо, ремонт штатных дхо спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S16" t="str">
+      <c r="U16" t="str">
         <v>Ремонт штатных ДХО в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T16" t="str">
+      <c r="V16" t="str">
         <v>Ремонт штатных ДХО в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1402,54 +1498,60 @@
         <v>4000</v>
       </c>
       <c r="D17" t="str">
+        <v>3-8 ч</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
         <v>Монтируем динамические поворотники с прошивкой или обманками при необходимости.</v>
       </c>
-      <c r="E17" t="str">
+      <c r="G17" t="str">
         <v>Динамика, Стильно</v>
       </c>
-      <c r="F17" t="str">
+      <c r="H17" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G17" t="str">
+      <c r="I17" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/MAAAgENOOA-19201.jpg</v>
       </c>
-      <c r="H17" t="str">
+      <c r="J17" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Установка / изготовление подсветки::от 4 000 ₽::3-8 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I17" t="str">
+      <c r="K17" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J17" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K17" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L17" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M17" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N17" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P17" t="str">
         <v>Сколько времени занимает установка динамических?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O17" t="str">
+      <c r="Q17" t="str">
         <v>динамические</v>
       </c>
-      <c r="P17" t="str">
+      <c r="R17" t="str">
         <v>Динамические («бегущие») поворотники в СПб — от 4 000 ₽ | К…</v>
       </c>
-      <c r="Q17" t="str">
+      <c r="S17" t="str">
         <v>Монтируем динамические поворотники с прошивкой или обманками при необходимости. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R17" t="str">
+      <c r="T17" t="str">
         <v>динамические, динамические спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S17" t="str">
+      <c r="U17" t="str">
         <v>Динамические («бегущие») поворотники в СПб — от 4 000 ₽ | К…</v>
       </c>
-      <c r="T17" t="str">
+      <c r="V17" t="str">
         <v>Динамические («бегущие») поворотники в СПб — от 4 000 ₽ | К…</v>
       </c>
     </row>
@@ -1464,54 +1566,60 @@
         <v>4000</v>
       </c>
       <c r="D18" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
         <v>Заменяем диоды в неразборных модулях — когда другим не по силам.</v>
       </c>
-      <c r="E18" t="str">
+      <c r="G18" t="str">
         <v>Редкие модели</v>
       </c>
-      <c r="F18" t="str">
+      <c r="H18" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G18" t="str">
+      <c r="I18" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/f01led.jpg</v>
       </c>
-      <c r="H18" t="str">
+      <c r="J18" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт светодиодных модулей::от 4 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I18" t="str">
+      <c r="K18" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J18" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K18" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L18" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M18" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N18" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P18" t="str">
         <v>Сколько времени занимает ремонт штатных светодиодных фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O18" t="str">
+      <c r="Q18" t="str">
         <v>ремонт светодиодных фар</v>
       </c>
-      <c r="P18" t="str">
+      <c r="R18" t="str">
         <v>Ремонт светодиодных фар (LED) в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q18" t="str">
+      <c r="S18" t="str">
         <v>Заменяем диоды в неразборных модулях — когда другим не по силам. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R18" t="str">
+      <c r="T18" t="str">
         <v>ремонт светодиодных фар, ремонт светодиодных фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S18" t="str">
+      <c r="U18" t="str">
         <v>Ремонт светодиодных фар (LED) в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T18" t="str">
+      <c r="V18" t="str">
         <v>Ремонт светодиодных фар (LED) в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1526,54 +1634,60 @@
         <v>3500</v>
       </c>
       <c r="D19" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
         <v>Восстанавливаем заднюю LED-оптику: диоды, платы, драйверы.</v>
       </c>
-      <c r="E19" t="str">
+      <c r="G19" t="str">
         <v>Задняя оптика</v>
       </c>
-      <c r="F19" t="str">
+      <c r="H19" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G19" t="str">
+      <c r="I19" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-9.jpg</v>
       </c>
-      <c r="H19" t="str">
+      <c r="J19" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт светодиодных модулей::от 3 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I19" t="str">
+      <c r="K19" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J19" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K19" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L19" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M19" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N19" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P19" t="str">
         <v>Сколько времени занимает ремонт штатных светодиодных фонарей?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O19" t="str">
+      <c r="Q19" t="str">
         <v>ремонт светодиодных фонарей</v>
       </c>
-      <c r="P19" t="str">
+      <c r="R19" t="str">
         <v>Ремонт светодиодных фонарей (задняя оптика) в СПб — от 3 50…</v>
       </c>
-      <c r="Q19" t="str">
+      <c r="S19" t="str">
         <v>Восстанавливаем заднюю LED-оптику: диоды, платы, драйверы. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R19" t="str">
+      <c r="T19" t="str">
         <v>ремонт светодиодных фонарей, ремонт светодиодных фонарей спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S19" t="str">
+      <c r="U19" t="str">
         <v>Ремонт светодиодных фонарей (задняя оптика) в СПб — от 3 50…</v>
       </c>
-      <c r="T19" t="str">
+      <c r="V19" t="str">
         <v>Ремонт светодиодных фонарей (задняя оптика) в СПб — от 3 50…</v>
       </c>
     </row>
@@ -1588,54 +1702,60 @@
         <v>6000</v>
       </c>
       <c r="D20" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
         <v>Монтаж ПТФ под ключ с прошивкой ЭБУ и активацией в меню.</v>
       </c>
-      <c r="E20" t="str">
+      <c r="G20" t="str">
         <v>Под ключ</v>
       </c>
-      <c r="F20" t="str">
+      <c r="H20" t="str">
         <v>Противотуманные фары (ПТФ)</v>
       </c>
-      <c r="G20" t="str">
+      <c r="I20" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/6f637804k444-19201.jpg</v>
       </c>
-      <c r="H20" t="str">
+      <c r="J20" t="str">
         <v>Установка ПТФ::от 6 000 ₽::2-4 ч::1 год|Программная активация (при необходимости)::входит в стоимость / от 2 000 ₽::+30-60 мин::-</v>
       </c>
-      <c r="I20" t="str">
+      <c r="K20" t="str">
         <v>Замена стекла / ламп ПТФ::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J20" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K20" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L20" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M20" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N20" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P20" t="str">
         <v>Сколько времени занимает установка и программная активация птф?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O20" t="str">
+      <c r="Q20" t="str">
         <v>установка и активация птф</v>
       </c>
-      <c r="P20" t="str">
+      <c r="R20" t="str">
         <v>Установка и активация ПТФ (с прошивкой ЭБУ) в СПб — от 6 00…</v>
       </c>
-      <c r="Q20" t="str">
+      <c r="S20" t="str">
         <v>Монтаж ПТФ под ключ с прошивкой ЭБУ и активацией в меню. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R20" t="str">
+      <c r="T20" t="str">
         <v>установка и активация птф, установка и активация птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S20" t="str">
+      <c r="U20" t="str">
         <v>Установка и активация ПТФ (с прошивкой ЭБУ) в СПб — от 6 00…</v>
       </c>
-      <c r="T20" t="str">
+      <c r="V20" t="str">
         <v>Установка и активация ПТФ (с прошивкой ЭБУ) в СПб — от 6 00…</v>
       </c>
     </row>
@@ -1650,54 +1770,60 @@
         <v>5000</v>
       </c>
       <c r="D21" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
         <v>Ставим LED ПТФ с правильной направленностью и подключением.</v>
       </c>
-      <c r="E21" t="str">
+      <c r="G21" t="str">
         <v>Яркий свет</v>
       </c>
-      <c r="F21" t="str">
+      <c r="H21" t="str">
         <v>Противотуманные фары (ПТФ)</v>
       </c>
-      <c r="G21" t="str">
+      <c r="I21" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/EAAAAgNVReA-19201.jpg</v>
       </c>
-      <c r="H21" t="str">
+      <c r="J21" t="str">
         <v>Установка ПТФ::от 5 000 ₽::2-4 ч::1 год|Программная активация (при необходимости)::входит в стоимость / от 2 000 ₽::+30-60 мин::-</v>
       </c>
-      <c r="I21" t="str">
+      <c r="K21" t="str">
         <v>Замена стекла / ламп ПТФ::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J21" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K21" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L21" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M21" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N21" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P21" t="str">
         <v>Сколько времени занимает установка светодиодных противотуманных фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O21" t="str">
+      <c r="Q21" t="str">
         <v>установка светодиодных птф</v>
       </c>
-      <c r="P21" t="str">
+      <c r="R21" t="str">
         <v>Установка светодиодных ПТФ в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q21" t="str">
+      <c r="S21" t="str">
         <v>Ставим LED ПТФ с правильной направленностью и подключением. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R21" t="str">
+      <c r="T21" t="str">
         <v>установка светодиодных птф, установка светодиодных птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S21" t="str">
+      <c r="U21" t="str">
         <v>Установка светодиодных ПТФ в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T21" t="str">
+      <c r="V21" t="str">
         <v>Установка светодиодных ПТФ в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1712,54 +1838,60 @@
         <v>3000</v>
       </c>
       <c r="D22" t="str">
+        <v>30-90 мин</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
         <v>Меняем треснувшее или мутное стекло ПТФ с герметизацией.</v>
       </c>
-      <c r="E22" t="str">
+      <c r="G22" t="str">
         <v>Герметично</v>
       </c>
-      <c r="F22" t="str">
+      <c r="H22" t="str">
         <v>Противотуманные фары (ПТФ)</v>
       </c>
-      <c r="G22" t="str">
+      <c r="I22" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/11/i-AAAgO2yeA-9601.jpg</v>
       </c>
-      <c r="H22" t="str">
+      <c r="J22" t="str">
         <v>Замена стёкол ПТФ::от 3 000 ₽::30-90 мин::6 мес.</v>
       </c>
-      <c r="I22" t="str">
+      <c r="K22" t="str">
         <v>Полировка стекла ПТФ::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J22" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K22" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L22" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M22" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N22" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P22" t="str">
         <v>Сколько времени занимает замена стёкол противотуманных фар?::Замена стёкол ПТФ — обычно до 1,5 часов.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
       </c>
-      <c r="O22" t="str">
+      <c r="Q22" t="str">
         <v>замена стёкол птф</v>
       </c>
-      <c r="P22" t="str">
+      <c r="R22" t="str">
         <v>Замена стёкол ПТФ в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q22" t="str">
+      <c r="S22" t="str">
         <v>Меняем треснувшее или мутное стекло ПТФ с герметизацией. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R22" t="str">
+      <c r="T22" t="str">
         <v>замена стёкол птф, замена стёкол птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S22" t="str">
+      <c r="U22" t="str">
         <v>Замена стёкол ПТФ в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T22" t="str">
+      <c r="V22" t="str">
         <v>Замена стёкол ПТФ в СПб — от 3 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1774,54 +1906,60 @@
         <v>1500</v>
       </c>
       <c r="D23" t="str">
+        <v>30-90 мин</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
         <v>Быстрая замена ламп в противотуманках с проверкой контактов.</v>
       </c>
-      <c r="E23" t="str">
+      <c r="G23" t="str">
         <v>Быстро</v>
       </c>
-      <c r="F23" t="str">
+      <c r="H23" t="str">
         <v>Противотуманные фары (ПТФ)</v>
       </c>
-      <c r="G23" t="str">
+      <c r="I23" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/6f637804k444-19201.jpg</v>
       </c>
-      <c r="H23" t="str">
+      <c r="J23" t="str">
         <v>Замена ламп в ПТФ::от 1 500 ₽::30-90 мин::-</v>
       </c>
-      <c r="I23" t="str">
+      <c r="K23" t="str">
         <v>Полировка стекла ПТФ::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J23" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K23" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L23" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M23" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N23" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P23" t="str">
         <v>Сколько времени занимает замена ламп в птф?::Работы занимают 30–90 минут.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 1 500 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
       </c>
-      <c r="O23" t="str">
+      <c r="Q23" t="str">
         <v>замена ламп в птф</v>
       </c>
-      <c r="P23" t="str">
+      <c r="R23" t="str">
         <v>Замена ламп в ПТФ в СПб — от 1 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q23" t="str">
+      <c r="S23" t="str">
         <v>Быстрая замена ламп в противотуманках с проверкой контактов. Цена от 1 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R23" t="str">
+      <c r="T23" t="str">
         <v>замена ламп в птф, замена ламп в птф спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S23" t="str">
+      <c r="U23" t="str">
         <v>Замена ламп в ПТФ в СПб — от 1 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T23" t="str">
+      <c r="V23" t="str">
         <v>Замена ламп в ПТФ в СПб — от 1 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -1836,54 +1974,60 @@
         <v>2000</v>
       </c>
       <c r="D24" t="str">
+        <v>30-90 мин</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
         <v>Переводим салон, габариты и подсветку номера на качественные LED.</v>
       </c>
-      <c r="E24" t="str">
+      <c r="G24" t="str">
         <v>Экономия энергии</v>
       </c>
-      <c r="F24" t="str">
+      <c r="H24" t="str">
         <v>Доп. услуги</v>
       </c>
-      <c r="G24" t="str">
+      <c r="I24" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/e53.jpg</v>
       </c>
-      <c r="H24" t="str">
+      <c r="J24" t="str">
         <v>Замена ламп на светодиодные::от 2 000 ₽::30-90 мин::1 год</v>
       </c>
-      <c r="I24" t="str">
+      <c r="K24" t="str">
         <v>Установка «обманок» (при ошибках в бортовом)::от 500 ₽::+15 мин::-</v>
       </c>
-      <c r="J24" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K24" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L24" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M24" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N24" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P24" t="str">
         <v>Сколько времени занимает замена ламп на светодиодные?::Замена ламп занимает от 30 минут.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
       </c>
-      <c r="O24" t="str">
+      <c r="Q24" t="str">
         <v>замена ламп на светодиодные</v>
       </c>
-      <c r="P24" t="str">
+      <c r="R24" t="str">
         <v>Замена ламп на светодиодные (салон, габариты, подсветка ном…</v>
       </c>
-      <c r="Q24" t="str">
+      <c r="S24" t="str">
         <v>Переводим салон, габариты и подсветку номера на качественные LED. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R24" t="str">
+      <c r="T24" t="str">
         <v>замена ламп на светодиодные, замена ламп на светодиодные спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S24" t="str">
+      <c r="U24" t="str">
         <v>Замена ламп на светодиодные (салон, габариты, подсветка ном…</v>
       </c>
-      <c r="T24" t="str">
+      <c r="V24" t="str">
         <v>Замена ламп на светодиодные (салон, габариты, подсветка ном…</v>
       </c>
     </row>
@@ -1898,54 +2042,60 @@
         <v>2500</v>
       </c>
       <c r="D25" t="str">
+        <v>1-3 ч</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
         <v>Чиним ручные и автоматические корректоры — мотор, тяги, датчики.</v>
       </c>
-      <c r="E25" t="str">
+      <c r="G25" t="str">
         <v>Ручной и авто</v>
       </c>
-      <c r="F25" t="str">
+      <c r="H25" t="str">
         <v>Механика</v>
       </c>
-      <c r="G25" t="str">
+      <c r="I25" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/sequoia-1.jpg</v>
       </c>
-      <c r="H25" t="str">
+      <c r="J25" t="str">
         <v>Диагностика узла::Входит в стоимость::30 мин::-|Ремонт механики::от 2 500 ₽::1-3 ч::1 год</v>
       </c>
-      <c r="I25" t="str">
+      <c r="K25" t="str">
         <v>Замена узла целиком::по согласованию::+1-2 ч::по запчасти</v>
       </c>
-      <c r="J25" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K25" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L25" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M25" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N25" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P25" t="str">
         <v>Сколько времени занимает ремонт корректора фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O25" t="str">
+      <c r="Q25" t="str">
         <v>ремонт корректора фар</v>
       </c>
-      <c r="P25" t="str">
+      <c r="R25" t="str">
         <v>Ремонт корректора фар (ручной/авто) в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="Q25" t="str">
+      <c r="S25" t="str">
         <v>Чиним ручные и автоматические корректоры — мотор, тяги, датчики. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R25" t="str">
+      <c r="T25" t="str">
         <v>ремонт корректора фар, ремонт корректора фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S25" t="str">
+      <c r="U25" t="str">
         <v>Ремонт корректора фар (ручной/авто) в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="T25" t="str">
+      <c r="V25" t="str">
         <v>Ремонт корректора фар (ручной/авто) в СПб — от 2 500 ₽ | КБ…</v>
       </c>
     </row>
@@ -1960,54 +2110,60 @@
         <v>2000</v>
       </c>
       <c r="D26" t="str">
+        <v>1-3 ч</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
         <v>Чистим форсунки, ремонтируем насосы и магистрали омывателя.</v>
       </c>
-      <c r="E26" t="str">
+      <c r="G26" t="str">
         <v>Форсунки, Насос</v>
       </c>
-      <c r="F26" t="str">
+      <c r="H26" t="str">
         <v>Механика</v>
       </c>
-      <c r="G26" t="str">
+      <c r="I26" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/08/IMG_toyota-nolden-pioneer-bixenon-1.jpg</v>
       </c>
-      <c r="H26" t="str">
+      <c r="J26" t="str">
         <v>Диагностика узла::Входит в стоимость::30 мин::-|Ремонт механики::от 2 000 ₽::1-3 ч::1 год</v>
       </c>
-      <c r="I26" t="str">
+      <c r="K26" t="str">
         <v>Замена узла целиком::по согласованию::+1-2 ч::по запчасти</v>
       </c>
-      <c r="J26" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K26" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L26" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M26" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N26" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P26" t="str">
         <v>Сколько времени занимает ремонт омывателя фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O26" t="str">
+      <c r="Q26" t="str">
         <v>ремонт омывателя фар</v>
       </c>
-      <c r="P26" t="str">
+      <c r="R26" t="str">
         <v>Ремонт омывателя фар в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q26" t="str">
+      <c r="S26" t="str">
         <v>Чистим форсунки, ремонтируем насосы и магистрали омывателя. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R26" t="str">
+      <c r="T26" t="str">
         <v>ремонт омывателя фар, ремонт омывателя фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S26" t="str">
+      <c r="U26" t="str">
         <v>Ремонт омывателя фар в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T26" t="str">
+      <c r="V26" t="str">
         <v>Ремонт омывателя фар в СПб — от 2 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2022,54 +2178,60 @@
         <v>6000</v>
       </c>
       <c r="D27" t="str">
+        <v>3-5 ч</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
         <v>Чистим, заменяем или восстанавливаем отражатели методом вакуумного напыления — как с завода.</v>
       </c>
-      <c r="E27" t="str">
+      <c r="G27" t="str">
         <v>Восстановление света</v>
       </c>
-      <c r="F27" t="str">
+      <c r="H27" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G27" t="str">
+      <c r="I27" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/reflector-1.png</v>
       </c>
-      <c r="H27" t="str">
+      <c r="J27" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Чистка или замена отражателей::от 6 000 ₽::3-5 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I27" t="str">
+      <c r="K27" t="str">
         <v>Вакуумное напыление отражателя::от 6 000 ₽::+1 день::1 год|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J27" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K27" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L27" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M27" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N27" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P27" t="str">
         <v>Сколько времени занимает ремонт отражателей фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O27" t="str">
+      <c r="Q27" t="str">
         <v>ремонт отражателей / вакуумное напыление</v>
       </c>
-      <c r="P27" t="str">
+      <c r="R27" t="str">
         <v>Ремонт отражателей / вакуумное напыление в СПб — от 6 000 ₽…</v>
       </c>
-      <c r="Q27" t="str">
+      <c r="S27" t="str">
         <v>Чистим, заменяем или восстанавливаем отражатели методом вакуумного напыления — как с завода. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R27" t="str">
+      <c r="T27" t="str">
         <v>ремонт отражателей / вакуумное напыление, ремонт отражателей / вакуумное напыление спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S27" t="str">
+      <c r="U27" t="str">
         <v>Ремонт отражателей / вакуумное напыление в СПб — от 6 000 ₽…</v>
       </c>
-      <c r="T27" t="str">
+      <c r="V27" t="str">
         <v>Ремонт отражателей / вакуумное напыление в СПб — от 6 000 ₽…</v>
       </c>
     </row>
@@ -2084,54 +2246,60 @@
         <v>2500</v>
       </c>
       <c r="D28" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
         <v>Герметично восстанавливаем трещины и сколы корпуса фары.</v>
       </c>
-      <c r="E28" t="str">
+      <c r="G28" t="str">
         <v>Герметичность</v>
       </c>
-      <c r="F28" t="str">
+      <c r="H28" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G28" t="str">
+      <c r="I28" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/9AAAAgDfYuA-19201.jpg</v>
       </c>
-      <c r="H28" t="str">
+      <c r="J28" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт корпуса фары::от 2 500 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I28" t="str">
+      <c r="K28" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J28" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K28" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L28" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M28" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N28" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P28" t="str">
         <v>Сколько времени занимает ремонт корпуса фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O28" t="str">
+      <c r="Q28" t="str">
         <v>ремонт корпуса фар</v>
       </c>
-      <c r="P28" t="str">
+      <c r="R28" t="str">
         <v>Ремонт корпуса фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q28" t="str">
+      <c r="S28" t="str">
         <v>Герметично восстанавливаем трещины и сколы корпуса фары. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R28" t="str">
+      <c r="T28" t="str">
         <v>ремонт корпуса фар, ремонт корпуса фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S28" t="str">
+      <c r="U28" t="str">
         <v>Ремонт корпуса фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T28" t="str">
+      <c r="V28" t="str">
         <v>Ремонт корпуса фар в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2146,54 +2314,60 @@
         <v>2500</v>
       </c>
       <c r="D29" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
         <v>Сварка пластика или ремкомплекты — фара снова держится надёжно.</v>
       </c>
-      <c r="E29" t="str">
+      <c r="G29" t="str">
         <v>Сварка пластика</v>
       </c>
-      <c r="F29" t="str">
+      <c r="H29" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G29" t="str">
+      <c r="I29" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/11/h0AAAgEVyeA-9601.jpg</v>
       </c>
-      <c r="H29" t="str">
+      <c r="J29" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Восстановление креплений («ушек»)::от 2 500 ₽::2-4 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I29" t="str">
+      <c r="K29" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J29" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K29" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L29" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M29" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N29" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O29" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P29" t="str">
         <v>Сколько времени занимает восстановление креплений?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O29" t="str">
+      <c r="Q29" t="str">
         <v>восстановление креплений</v>
       </c>
-      <c r="P29" t="str">
+      <c r="R29" t="str">
         <v>Восстановление креплений («ушек») в СПб — от 2 500 ₽ | КБ А…</v>
       </c>
-      <c r="Q29" t="str">
+      <c r="S29" t="str">
         <v>Сварка пластика или ремкомплекты — фара снова держится надёжно. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R29" t="str">
+      <c r="T29" t="str">
         <v>восстановление креплений, восстановление креплений спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S29" t="str">
+      <c r="U29" t="str">
         <v>Восстановление креплений («ушек») в СПб — от 2 500 ₽ | КБ А…</v>
       </c>
-      <c r="T29" t="str">
+      <c r="V29" t="str">
         <v>Восстановление креплений («ушек») в СПб — от 2 500 ₽ | КБ А…</v>
       </c>
     </row>
@@ -2208,54 +2382,60 @@
         <v>3000</v>
       </c>
       <c r="D30" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
         <v>Диагностика и ремонт специфических узлов штатного ксенона.</v>
       </c>
-      <c r="E30" t="str">
+      <c r="G30" t="str">
         <v>Штатный ксенон</v>
       </c>
-      <c r="F30" t="str">
+      <c r="H30" t="str">
         <v>Механика</v>
       </c>
-      <c r="G30" t="str">
+      <c r="I30" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/m37-1.jpg</v>
       </c>
-      <c r="H30" t="str">
+      <c r="J30" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 3 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I30" t="str">
+      <c r="K30" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J30" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K30" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L30" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M30" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N30" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P30" t="str">
         <v>Сколько времени занимает ремонт ксеноновых фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O30" t="str">
+      <c r="Q30" t="str">
         <v>ремонт ксеноновых фар</v>
       </c>
-      <c r="P30" t="str">
+      <c r="R30" t="str">
         <v>Ремонт ксеноновых фар (спец. узлы) в СПб — от 3 000 ₽ | КБ…</v>
       </c>
-      <c r="Q30" t="str">
+      <c r="S30" t="str">
         <v>Диагностика и ремонт специфических узлов штатного ксенона. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R30" t="str">
+      <c r="T30" t="str">
         <v>ремонт ксеноновых фар, ремонт ксеноновых фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S30" t="str">
+      <c r="U30" t="str">
         <v>Ремонт ксеноновых фар (спец. узлы) в СПб — от 3 000 ₽ | КБ…</v>
       </c>
-      <c r="T30" t="str">
+      <c r="V30" t="str">
         <v>Ремонт ксеноновых фар (спец. узлы) в СПб — от 3 000 ₽ | КБ…</v>
       </c>
     </row>
@@ -2270,54 +2450,60 @@
         <v>5000</v>
       </c>
       <c r="D31" t="str">
+        <v>2-3 ч</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
         <v>Подбираем оптимальное решение под ваш бюджет и задачи.</v>
       </c>
-      <c r="E31" t="str">
+      <c r="G31" t="str">
         <v>Под ваш бюджет</v>
       </c>
-      <c r="F31" t="str">
+      <c r="H31" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G31" t="str">
+      <c r="I31" t="str">
         <v>https://ksenonspb.ru/portfolio/7MAAAgAzWOA-1920.jpg</v>
       </c>
-      <c r="H31" t="str">
+      <c r="J31" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Замена линз Bi-LED / Xenon::от 5 000 ₽ / шт.::2-3 ч::2 года|Калибровка светового пучка::входит в стоимость::30 мин::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I31" t="str">
+      <c r="K31" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J31" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K31" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L31" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M31" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N31" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P31" t="str">
         <v>Сколько времени занимает комплексное улучшение света фар?::Базовые работы по линзам — обычно 2–4 часа на фару.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O31" t="str">
+      <c r="Q31" t="str">
         <v>комплексное улучшение света</v>
       </c>
-      <c r="P31" t="str">
+      <c r="R31" t="str">
         <v>Комплексное улучшение света в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q31" t="str">
+      <c r="S31" t="str">
         <v>Подбираем оптимальное решение под ваш бюджет и задачи. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R31" t="str">
+      <c r="T31" t="str">
         <v>комплексное улучшение света, комплексное улучшение света спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S31" t="str">
+      <c r="U31" t="str">
         <v>Комплексное улучшение света в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T31" t="str">
+      <c r="V31" t="str">
         <v>Комплексное улучшение света в СПб — от 5 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2332,54 +2518,60 @@
         <v>3500</v>
       </c>
       <c r="D32" t="str">
+        <v>от 2 ч</v>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
         <v>Ремонт и восстановление фар европейских брендов — Valeo, Hella, Bosch, Magneti Marelli и аналоги.</v>
       </c>
-      <c r="E32" t="str">
+      <c r="G32" t="str">
         <v>Опыт с европейской оптикой</v>
       </c>
-      <c r="F32" t="str">
+      <c r="H32" t="str">
         <v>Ремонт фар</v>
       </c>
-      <c r="G32" t="str">
+      <c r="I32" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/16c6149s-960.jpg</v>
       </c>
-      <c r="H32" t="str">
+      <c r="J32" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 3 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I32" t="str">
+      <c r="K32" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J32" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K32" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L32" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="N32" t="str">
         <v>BMW|MERCEDES|AUDI|Volkswagen|PORSCHE|VOLVO|Land Rover|JAGUAR|MINI|Skoda|OPEL|PEUGEOT|RENAULT</v>
       </c>
-      <c r="M32" t="str">
-        <v>Частые вопросы</v>
-      </c>
-      <c r="N32" t="str">
+      <c r="O32" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P32" t="str">
         <v>Сколько времени занимает ремонт фар европейских производителей?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O32" t="str">
+      <c r="Q32" t="str">
         <v>ремонт фар европейских производителей</v>
       </c>
-      <c r="P32" t="str">
+      <c r="R32" t="str">
         <v>Ремонт фар европейских производителей в СПб — от 3 500 ₽ |…</v>
       </c>
-      <c r="Q32" t="str">
+      <c r="S32" t="str">
         <v>Ремонт и восстановление фар европейских брендов — Valeo, Hella, Bosch, Magneti Marelli и аналоги. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R32" t="str">
+      <c r="T32" t="str">
         <v>ремонт фар европейских производителей, ремонт фар европейских производителей спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S32" t="str">
+      <c r="U32" t="str">
         <v>Ремонт фар европейских производителей в СПб — от 3 500 ₽ |…</v>
       </c>
-      <c r="T32" t="str">
+      <c r="V32" t="str">
         <v>Ремонт фар европейских производителей в СПб — от 3 500 ₽ |…</v>
       </c>
     </row>
@@ -2394,54 +2586,60 @@
         <v>2500</v>
       </c>
       <c r="D33" t="str">
+        <v>от 2 ч</v>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
         <v>Восстанавливаем фары китайских марок — часто неразборные LED-модули и нестандартная геометрия.</v>
       </c>
-      <c r="E33" t="str">
+      <c r="G33" t="str">
         <v>Неразборные модули</v>
       </c>
-      <c r="F33" t="str">
+      <c r="H33" t="str">
         <v>Ремонт фар</v>
       </c>
-      <c r="G33" t="str">
+      <c r="I33" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/11/KFAAAgLSoeA-9601.jpg</v>
       </c>
-      <c r="H33" t="str">
+      <c r="J33" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 2 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I33" t="str">
+      <c r="K33" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J33" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K33" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L33" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="N33" t="str">
         <v>TOYOTA|LEXUS|NISSAN|HONDA|MAZDA|MITSUBISHI|SUBARU|SUZUKI|KIA|Hyundai|INFINITI|SsangYong</v>
       </c>
-      <c r="M33" t="str">
-        <v>Частые вопросы</v>
-      </c>
-      <c r="N33" t="str">
+      <c r="O33" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P33" t="str">
         <v>Сколько времени занимает ремонт фар китайских производителей?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O33" t="str">
+      <c r="Q33" t="str">
         <v>ремонт фар китайских производителей</v>
       </c>
-      <c r="P33" t="str">
+      <c r="R33" t="str">
         <v>Ремонт фар китайских производителей в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="Q33" t="str">
+      <c r="S33" t="str">
         <v>Восстанавливаем фары китайских марок — часто неразборные LED-модули и нестандартная геометрия. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R33" t="str">
+      <c r="T33" t="str">
         <v>ремонт фар китайских производителей, ремонт фар китайских производителей спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S33" t="str">
+      <c r="U33" t="str">
         <v>Ремонт фар китайских производителей в СПб — от 2 500 ₽ | КБ…</v>
       </c>
-      <c r="T33" t="str">
+      <c r="V33" t="str">
         <v>Ремонт фар китайских производителей в СПб — от 2 500 ₽ | КБ…</v>
       </c>
     </row>
@@ -2456,54 +2654,60 @@
         <v>3500</v>
       </c>
       <c r="D34" t="str">
+        <v>от 2 ч</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
         <v>Ремонт оптики американского рынка — отличия в креплениях, проводке и светораспределении.</v>
       </c>
-      <c r="E34" t="str">
+      <c r="G34" t="str">
         <v>Специфика USDM</v>
       </c>
-      <c r="F34" t="str">
+      <c r="H34" t="str">
         <v>Ремонт фар</v>
       </c>
-      <c r="G34" t="str">
+      <c r="I34" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/BYAAAgOQwuA-19201.jpg</v>
       </c>
-      <c r="H34" t="str">
+      <c r="J34" t="str">
         <v>Диагностика и оценка объёма работ::Входит в стоимость::30 мин::-|Ремонт / восстановление фары::от 3 500 ₽::от 2 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I34" t="str">
+      <c r="K34" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J34" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K34" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L34" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="N34" t="str">
         <v>FORD|CHEVROLET|CADILLAC|JEEP|DODGE|CHRYSLER|HUMMER|ACURA</v>
       </c>
-      <c r="M34" t="str">
-        <v>Частые вопросы</v>
-      </c>
-      <c r="N34" t="str">
+      <c r="O34" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P34" t="str">
         <v>Сколько времени занимает ремонт фар американского рынка?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O34" t="str">
+      <c r="Q34" t="str">
         <v>ремонт фар американского рынка</v>
       </c>
-      <c r="P34" t="str">
+      <c r="R34" t="str">
         <v>Ремонт фар американского рынка в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q34" t="str">
+      <c r="S34" t="str">
         <v>Ремонт оптики американского рынка — отличия в креплениях, проводке и светораспределении. Цена от 3 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R34" t="str">
+      <c r="T34" t="str">
         <v>ремонт фар американского рынка, ремонт фар американского рынка спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S34" t="str">
+      <c r="U34" t="str">
         <v>Ремонт фар американского рынка в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T34" t="str">
+      <c r="V34" t="str">
         <v>Ремонт фар американского рынка в СПб — от 3 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2518,54 +2722,60 @@
         <v>4000</v>
       </c>
       <c r="D35" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
         <v>Диагностика и ремонт AFS: моторы, датчики, блоки управления.</v>
       </c>
-      <c r="E35" t="str">
+      <c r="G35" t="str">
         <v>AFS, Адаптивный свет</v>
       </c>
-      <c r="F35" t="str">
+      <c r="H35" t="str">
         <v>Регулировка и диагностика</v>
       </c>
-      <c r="G35" t="str">
+      <c r="I35" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/b6ceb9ds-960.jpg</v>
       </c>
-      <c r="H35" t="str">
+      <c r="J35" t="str">
         <v>Диагностика системы AFS::Входит в стоимость::30-60 мин::-|Ремонт / адаптация AFS::от 4 000 ₽::2-6 ч::1 год</v>
       </c>
-      <c r="I35" t="str">
+      <c r="K35" t="str">
         <v>Замена датчиков / блоков::по согласованию::+2-4 ч::по запчасти</v>
       </c>
-      <c r="J35" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K35" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L35" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="N35" t="str">
         <v>BMW|MERCEDES|AUDI|LEXUS|PORSCHE|Land Rover|JAGUAR|INFINITI|Maserati|BENTLEY</v>
       </c>
-      <c r="M35" t="str">
-        <v>Частые вопросы</v>
-      </c>
-      <c r="N35" t="str">
+      <c r="O35" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P35" t="str">
         <v>Сколько времени занимает ремонт систем адаптивного освещения?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O35" t="str">
+      <c r="Q35" t="str">
         <v>ремонт систем адаптивного освещения</v>
       </c>
-      <c r="P35" t="str">
+      <c r="R35" t="str">
         <v>Ремонт систем адаптивного освещения (AFS) в СПб — от 4 000…</v>
       </c>
-      <c r="Q35" t="str">
+      <c r="S35" t="str">
         <v>Диагностика и ремонт AFS: моторы, датчики, блоки управления. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R35" t="str">
+      <c r="T35" t="str">
         <v>ремонт систем адаптивного освещения, ремонт систем адаптивного освещения спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S35" t="str">
+      <c r="U35" t="str">
         <v>Ремонт систем адаптивного освещения (AFS) в СПб — от 4 000…</v>
       </c>
-      <c r="T35" t="str">
+      <c r="V35" t="str">
         <v>Ремонт систем адаптивного освещения (AFS) в СПб — от 4 000…</v>
       </c>
     </row>
@@ -2580,54 +2790,60 @@
         <v>6000</v>
       </c>
       <c r="D36" t="str">
+        <v>1-2 дня</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
         <v>Восстанавливаем выгоревшие отражатели методом вакуумного напыления — заводское качество отражения.</v>
       </c>
-      <c r="E36" t="str">
+      <c r="G36" t="str">
         <v>Как с завода</v>
       </c>
-      <c r="F36" t="str">
+      <c r="H36" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G36" t="str">
+      <c r="I36" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/reflector-1.png</v>
       </c>
-      <c r="H36" t="str">
+      <c r="J36" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Вакуумное напыление отражателей::от 6 000 ₽::1-2 дня::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I36" t="str">
+      <c r="K36" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J36" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K36" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L36" t="str">
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
+      </c>
+      <c r="N36" t="str">
         <v>BMW|MERCEDES|AUDI|LEXUS|PORSCHE|Land Rover|JAGUAR|INFINITI|Maserati|BENTLEY</v>
       </c>
-      <c r="M36" t="str">
-        <v>Частые вопросы</v>
-      </c>
-      <c r="N36" t="str">
+      <c r="O36" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P36" t="str">
         <v>Сколько времени занимает восстановление отражателей методом вакуумного напыления?::Вакуумное напыление занимает 1–2 рабочих дня.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 6 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O36" t="str">
+      <c r="Q36" t="str">
         <v>восстановление отражателей методом вакуумного напыления</v>
       </c>
-      <c r="P36" t="str">
+      <c r="R36" t="str">
         <v>Восстановление отражателей методом вакуумного напыления в С…</v>
       </c>
-      <c r="Q36" t="str">
+      <c r="S36" t="str">
         <v>Восстанавливаем выгоревшие отражатели методом вакуумного напыления — заводское качество отражения. Цена от 6 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R36" t="str">
+      <c r="T36" t="str">
         <v>восстановление отражателей методом вакуумного напыления, восстановление отражателей методом вакуумного напыления спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S36" t="str">
+      <c r="U36" t="str">
         <v>Восстановление отражателей методом вакуумного напыления в С…</v>
       </c>
-      <c r="T36" t="str">
+      <c r="V36" t="str">
         <v>Восстановление отражателей методом вакуумного напыления в С…</v>
       </c>
     </row>
@@ -2642,54 +2858,60 @@
         <v>4000</v>
       </c>
       <c r="D37" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
         <v>Перепаиваем LED-драйверы и платы управления в фарах и фонарях.</v>
       </c>
-      <c r="E37" t="str">
+      <c r="G37" t="str">
         <v>Электроника</v>
       </c>
-      <c r="F37" t="str">
+      <c r="H37" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G37" t="str">
+      <c r="I37" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2020/03/SGAAAgIfOeA-19201.jpg</v>
       </c>
-      <c r="H37" t="str">
+      <c r="J37" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт / перепайка платы::от 4 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I37" t="str">
+      <c r="K37" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J37" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K37" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L37" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M37" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N37" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P37" t="str">
         <v>Сколько времени занимает ремонт и перепайка драйверов?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O37" t="str">
+      <c r="Q37" t="str">
         <v>ремонт/перепайка драйверов</v>
       </c>
-      <c r="P37" t="str">
+      <c r="R37" t="str">
         <v>Ремонт/перепайка драйверов (плат) LED в СПб — от 4 000 ₽ |…</v>
       </c>
-      <c r="Q37" t="str">
+      <c r="S37" t="str">
         <v>Перепаиваем LED-драйверы и платы управления в фарах и фонарях. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R37" t="str">
+      <c r="T37" t="str">
         <v>ремонт/перепайка драйверов, ремонт/перепайка драйверов спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S37" t="str">
+      <c r="U37" t="str">
         <v>Ремонт/перепайка драйверов (плат) LED в СПб — от 4 000 ₽ |…</v>
       </c>
-      <c r="T37" t="str">
+      <c r="V37" t="str">
         <v>Ремонт/перепайка драйверов (плат) LED в СПб — от 4 000 ₽ |…</v>
       </c>
     </row>
@@ -2704,54 +2926,60 @@
         <v>5000</v>
       </c>
       <c r="D38" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
         <v>Ремонт и прошивка блоков управления фарой.</v>
       </c>
-      <c r="E38" t="str">
+      <c r="G38" t="str">
         <v>ЭБУ фары</v>
       </c>
-      <c r="F38" t="str">
+      <c r="H38" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G38" t="str">
+      <c r="I38" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/e-repair-1.jpg</v>
       </c>
-      <c r="H38" t="str">
+      <c r="J38" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт / перепайка платы::от 5 000 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I38" t="str">
+      <c r="K38" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J38" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K38" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L38" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M38" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N38" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P38" t="str">
         <v>Сколько времени занимает ремонт контроллеров управления фарой?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 5 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O38" t="str">
+      <c r="Q38" t="str">
         <v>ремонт контроллеров управления фарой</v>
       </c>
-      <c r="P38" t="str">
+      <c r="R38" t="str">
         <v>Ремонт контроллеров управления фарой (ЭБУ) в СПб — от 5 000…</v>
       </c>
-      <c r="Q38" t="str">
+      <c r="S38" t="str">
         <v>Ремонт и прошивка блоков управления фарой. Цена от 5 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R38" t="str">
+      <c r="T38" t="str">
         <v>ремонт контроллеров управления фарой, ремонт контроллеров управления фарой спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S38" t="str">
+      <c r="U38" t="str">
         <v>Ремонт контроллеров управления фарой (ЭБУ) в СПб — от 5 000…</v>
       </c>
-      <c r="T38" t="str">
+      <c r="V38" t="str">
         <v>Ремонт контроллеров управления фарой (ЭБУ) в СПб — от 5 000…</v>
       </c>
     </row>
@@ -2766,54 +2994,60 @@
         <v>2500</v>
       </c>
       <c r="D39" t="str">
+        <v>2-3 ч</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
         <v>Удаляем налёт и помутнение изнутри фары без разборки корпуса.</v>
       </c>
-      <c r="E39" t="str">
+      <c r="G39" t="str">
         <v>Без разборки</v>
       </c>
-      <c r="F39" t="str">
+      <c r="H39" t="str">
         <v>Оптика и корпус</v>
       </c>
-      <c r="G39" t="str">
+      <c r="I39" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/cleaning-1.jpg</v>
       </c>
-      <c r="H39" t="str">
+      <c r="J39" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Химическая чистка изнутри::от 2 500 ₽::2-3 ч::-|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I39" t="str">
+      <c r="K39" t="str">
         <v>Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-|Покраска масок и декоративных элементов::от 2 000 ₽::+1 день::-</v>
       </c>
-      <c r="J39" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K39" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L39" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M39" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N39" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P39" t="str">
         <v>Сколько времени занимает химическая чистка фары изнутри?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O39" t="str">
+      <c r="Q39" t="str">
         <v>химчистка фары изнутри</v>
       </c>
-      <c r="P39" t="str">
+      <c r="R39" t="str">
         <v>Химчистка фары изнутри в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q39" t="str">
+      <c r="S39" t="str">
         <v>Удаляем налёт и помутнение изнутри фары без разборки корпуса. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R39" t="str">
+      <c r="T39" t="str">
         <v>химчистка фары изнутри, химчистка фары изнутри спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S39" t="str">
+      <c r="U39" t="str">
         <v>Химчистка фары изнутри в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T39" t="str">
+      <c r="V39" t="str">
         <v>Химчистка фары изнутри в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2828,54 +3062,60 @@
         <v>2000</v>
       </c>
       <c r="D40" t="str">
+        <v>1-2 ч</v>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
         <v>Кодируем ЭБУ или ставим обманки — без ошибок на панели.</v>
       </c>
-      <c r="E40" t="str">
+      <c r="G40" t="str">
         <v>Без ошибок</v>
       </c>
-      <c r="F40" t="str">
+      <c r="H40" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G40" t="str">
+      <c r="I40" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2018/05/tmp-23.jpg</v>
       </c>
-      <c r="H40" t="str">
+      <c r="J40" t="str">
         <v>Компьютерная диагностика::Входит в стоимость::30 мин::-|Кодирование / программирование::от 2 000 ₽::1-2 ч::-</v>
       </c>
-      <c r="I40" t="str">
+      <c r="K40" t="str">
         <v>Установка «обманок» (при необходимости)::от 1 500 ₽::+30 мин::1 год</v>
       </c>
-      <c r="J40" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K40" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L40" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M40" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N40" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P40" t="str">
         <v>Сколько времени занимает программное отключение опроса ламп?::Диагностика и кодирование — обычно 1–2 часа.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
       </c>
-      <c r="O40" t="str">
+      <c r="Q40" t="str">
         <v>программное отключение опроса ламп</v>
       </c>
-      <c r="P40" t="str">
+      <c r="R40" t="str">
         <v>Программное отключение опроса ламп («обманки») в СПб — от 2…</v>
       </c>
-      <c r="Q40" t="str">
+      <c r="S40" t="str">
         <v>Кодируем ЭБУ или ставим обманки — без ошибок на панели. Цена от 2 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R40" t="str">
+      <c r="T40" t="str">
         <v>программное отключение опроса ламп, программное отключение опроса ламп спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S40" t="str">
+      <c r="U40" t="str">
         <v>Программное отключение опроса ламп («обманки») в СПб — от 2…</v>
       </c>
-      <c r="T40" t="str">
+      <c r="V40" t="str">
         <v>Программное отключение опроса ламп («обманки») в СПб — от 2…</v>
       </c>
     </row>
@@ -2890,54 +3130,60 @@
         <v>2500</v>
       </c>
       <c r="D41" t="str">
+        <v>2-6 ч</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
         <v>Меняем перегоревшую или повреждённую проводку внутри фары.</v>
       </c>
-      <c r="E41" t="str">
+      <c r="G41" t="str">
         <v>Надёжный контакт</v>
       </c>
-      <c r="F41" t="str">
+      <c r="H41" t="str">
         <v>Электрика и электроника</v>
       </c>
-      <c r="G41" t="str">
+      <c r="I41" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2021/09/5D7ZL-EXgUe6NbclWgUam9SMyS0-9601.jpg</v>
       </c>
-      <c r="H41" t="str">
+      <c r="J41" t="str">
         <v>Демонтаж фары и разборка корпуса::Входит в стоимость::1-2 ч::-|Ремонт электрики фары::от 2 500 ₽::2-6 ч::1 год|Герметизация и сборка::входит в стоимость::1 ч::1 год</v>
       </c>
-      <c r="I41" t="str">
+      <c r="K41" t="str">
         <v>Замена блоков / модулей (при необходимости)::по прайсу запчастей::+1-2 ч::по запчасти|Полировка стекла изнутри::от 1 500 ₽::+1 ч::1 год|Замена уплотнителя корпуса::от 800 ₽::+30 мин::-</v>
       </c>
-      <c r="J41" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K41" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L41" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M41" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N41" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O41" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P41" t="str">
         <v>Сколько времени занимает замена внутренней проводки фары?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 2 500 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O41" t="str">
+      <c r="Q41" t="str">
         <v>замена внутренней проводки фары</v>
       </c>
-      <c r="P41" t="str">
+      <c r="R41" t="str">
         <v>Замена внутренней проводки фары в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q41" t="str">
+      <c r="S41" t="str">
         <v>Меняем перегоревшую или повреждённую проводку внутри фары. Цена от 2 500 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R41" t="str">
+      <c r="T41" t="str">
         <v>замена внутренней проводки фары, замена внутренней проводки фары спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S41" t="str">
+      <c r="U41" t="str">
         <v>Замена внутренней проводки фары в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
-      <c r="T41" t="str">
+      <c r="V41" t="str">
         <v>Замена внутренней проводки фары в СПб — от 2 500 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -2952,54 +3198,60 @@
         <v>4000</v>
       </c>
       <c r="D42" t="str">
+        <v>2-4 ч</v>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
         <v>Монтируем автокорректоры с подключением к штатной системе.</v>
       </c>
-      <c r="E42" t="str">
+      <c r="G42" t="str">
         <v>Автокорректор</v>
       </c>
-      <c r="F42" t="str">
+      <c r="H42" t="str">
         <v>Тюнинг фар</v>
       </c>
-      <c r="G42" t="str">
+      <c r="I42" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2021/09/IKgT7yLzjx-1W7XenovHwM91Iys-960.jpg</v>
       </c>
-      <c r="H42" t="str">
+      <c r="J42" t="str">
         <v>Установка автокорректора::от 4 000 ₽::2-4 ч::1 год|Калибровка светового пучка::входит в стоимость::30 мин::-</v>
       </c>
-      <c r="I42" t="str">
+      <c r="K42" t="str">
         <v>Адаптация / кодирование::от 2 000 ₽::+1 ч::-</v>
       </c>
-      <c r="J42" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K42" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L42" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M42" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N42" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O42" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P42" t="str">
         <v>Сколько времени занимает установка автокорректоров фар?::Срок зависит от объёма работ; точное время скажем после осмотра.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 4 000 ₽.|Нужна ли разборка фары?::В большинстве случаев да — для качественного результата фару снимаем и разбираем. Демонтаж обычно входит в стоимость основных работ.</v>
       </c>
-      <c r="O42" t="str">
+      <c r="Q42" t="str">
         <v>установка автокорректоров фар</v>
       </c>
-      <c r="P42" t="str">
+      <c r="R42" t="str">
         <v>Установка автокорректоров фар в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="Q42" t="str">
+      <c r="S42" t="str">
         <v>Монтируем автокорректоры с подключением к штатной системе. Цена от 4 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R42" t="str">
+      <c r="T42" t="str">
         <v>установка автокорректоров фар, установка автокорректоров фар спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S42" t="str">
+      <c r="U42" t="str">
         <v>Установка автокорректоров фар в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
-      <c r="T42" t="str">
+      <c r="V42" t="str">
         <v>Установка автокорректоров фар в СПб — от 4 000 ₽ | КБ АВТО</v>
       </c>
     </row>
@@ -3014,60 +3266,66 @@
         <v>3000</v>
       </c>
       <c r="D43" t="str">
+        <v>1-2 ч</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
         <v>Кодируем блоки света, активируем функции, проводим компьютерную диагностику.</v>
       </c>
-      <c r="E43" t="str">
+      <c r="G43" t="str">
         <v>Диагностика, Кодирование</v>
       </c>
-      <c r="F43" t="str">
+      <c r="H43" t="str">
         <v>Регулировка и диагностика</v>
       </c>
-      <c r="G43" t="str">
+      <c r="I43" t="str">
         <v>https://ksenonspb.ru/wp-content/uploads/2016/09/e-repair-1.jpg</v>
       </c>
-      <c r="H43" t="str">
+      <c r="J43" t="str">
         <v>Компьютерная диагностика::Входит в стоимость::30 мин::-|Кодирование / программирование::от 3 000 ₽::1-2 ч::-</v>
       </c>
-      <c r="I43" t="str">
+      <c r="K43" t="str">
         <v>Установка «обманок» (при необходимости)::от 1 500 ₽::+30 мин::1 год</v>
       </c>
-      <c r="J43" t="str">
-        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
-      </c>
-      <c r="K43" t="str">
-        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
-      </c>
       <c r="L43" t="str">
-        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+        <v>Осмотр и заключение по фаре::Бесплатно::30 мин::-</v>
       </c>
       <c r="M43" t="str">
-        <v>Частые вопросы</v>
+        <v>Гарантия распространяется на установленные компоненты и герметизацию. Предоплата не требуется. Все работы фиксируются в договоре — вы забираете автомобиль с письменной гарантией.</v>
       </c>
       <c r="N43" t="str">
+        <v>BMW|MERCEDES|AUDI|TOYOTA|LEXUS|Volkswagen|KIA|Hyundai|NISSAN|FORD|HONDA|MAZDA|Skoda|Land Rover</v>
+      </c>
+      <c r="O43" t="str">
+        <v>Частые вопросы</v>
+      </c>
+      <c r="P43" t="str">
         <v>Сколько времени занимает кодирование и программирование штатных блоков управления светом + компьютерная диагностика?::Диагностика и кодирование — обычно 1–2 часа.|Какая гарантия на работы?::На установленные компоненты и герметизацию даём письменную гарантию. Срок по позициям указан в таблице цен.|Нужна ли предварительная запись?::Да, работы выполняем по записи. Осмотр и заключение по фаре — бесплатно.|От чего зависит итоговая цена?::На стоимость влияют состояние оптики, марка и модель автомобиля, а также дополнительные работы (полировка изнутри, уплотнители и т.п.). Ориентир по цене — от 3 000 ₽.|Нужна ли разборка фары?::Разборка фары обычно не требуется. Если по результатам осмотра она понадобится — согласуем заранее.</v>
       </c>
-      <c r="O43" t="str">
+      <c r="Q43" t="str">
         <v>кодирование/программирование блоков + диагностика</v>
       </c>
-      <c r="P43" t="str">
+      <c r="R43" t="str">
         <v>Кодирование/программирование блоков + диагностика в СПб — о…</v>
       </c>
-      <c r="Q43" t="str">
+      <c r="S43" t="str">
         <v>Кодируем блоки света, активируем функции, проводим компьютерную диагностику. Цена от 3 000 ₽. КБ АВТО, Санкт-Петербург.</v>
       </c>
-      <c r="R43" t="str">
+      <c r="T43" t="str">
         <v>кодирование/программирование блоков + диагностика, кодирование/программирование блоков + диагностика спб, ремонт фар СПб, тюнинг оптики СПб, КБ АВТО</v>
       </c>
-      <c r="S43" t="str">
+      <c r="U43" t="str">
         <v>Кодирование/программирование блоков + диагностика в СПб — о…</v>
       </c>
-      <c r="T43" t="str">
+      <c r="V43" t="str">
         <v>Кодирование/программирование блоков + диагностика в СПб — о…</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>